<commit_message>
chore: update question bank workbook
</commit_message>
<xml_diff>
--- a/data/Ngan-Hang-Cau-Hoi.xlsx
+++ b/data/Ngan-Hang-Cau-Hoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f54d0bdb7235122/Documents/My App/trac-nghiem-luat-dau-thau/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B32B0D1-E964-45B5-876C-751CC32868FC}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9945B2BA-DA03-453F-91C4-0EF789E4D547}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0822E189-CD53-41B9-B216-EFA7EF505EBC}"/>
   </bookViews>
@@ -1536,13 +1536,6 @@
 D. Đánh giá năng lực, kinh nghiệm của nhà thầu phụ căn cứ theo phần công việc nhà thầu phụ đảm nhận, nhà thầu tham dự thầu cũng phải đáp ứng về năng lực, kinh nghiệm đối với phần công việc mà nhà thầu phụ đảm nhận</t>
   </si>
   <si>
-    <t>A. Phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó để sửa đổi cho phù hợp và tiến hành nộp lại
-E-HSDT mới
-B. Không phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó, chỉ cần sửa đổi cho phù hợp và tiến hành nộp lại E-HSDT mới
-C. Sửa đổi cho phù hợp E-HSDT đã nộp mà không phải nộp lại E- HSDT mới
-D. Các phương án trên đều sai</t>
-  </si>
-  <si>
     <t>Đối với đấu thầu qua mạng, trường hợp nhà thầu rút E-HSDT sau thời điểm đóng thầu và trong thời gian có hiệu lực của E-HSDT thì
 nhà thầu bị xử lý theo phương án nào sau đây?</t>
   </si>
@@ -3782,13 +3775,6 @@
 D. Phải đảm bảo tổng số lượng hàng hóa mà các nhà thầu trúng thầu chào thầu bằng số lượng hàng hóa nêu trong hồ sơ mời thầu, đồng thời bảo đảm tổng giá đánh giá của gói thầu là thấp nhất</t>
   </si>
   <si>
-    <t>A. Cấm tham gia hoạt động đấu thầu từ 03 năm đến 05 năm đối với thành viên A
-B. Cấm tham gia hoạt động đấu thầu từ 01 năm đến dưới 03 năm đối với thành viên A
-C. Cấm tham gia hoạt động đấu thầu từ 03 năm đến 05 năm đối với tất cả thành viên trong nhà thầu liên danh A-B
-D. Cấm tham gia hoạt động đấu thầu từ 01 năm đến 03 năm đối với tất cả thành viên trong nhà thầu
-liên danh A-B</t>
-  </si>
-  <si>
     <t>A. Từ ngày có thời điểm đóng thầu đến khi có kết quả lựa chọn nhà thầu
 B. Từ ngày phát hành hồ sơ mời sơ tuyển, hồ sơ mời quan tâm, hồ sơ mời thầu, hồ sơ yêu cầu đến trước khi ký kết hợp đồng, thỏa thuận khung đối với mua sắm tập trung
 C. Từ ngày có thời điểm đóng thầu đến khi ký kết hợp đồng, thỏa thuận khung đối với mua sắm tập trung
@@ -3801,13 +3787,6 @@
 D. Nhà thầu đã hoàn thành công trình xây dựng nhà, kết cấu dạng nhà cấp III, có giá trị tối thiểu là 50% x (2X) VND, trong đó phải bao gồm hạng mục hàng rào bảo vệ, nhà bảo vệ</t>
   </si>
   <si>
-    <t>A. Chủ đầu tư phải ghi tỷ lệ % giá trị dành cho nhà thầu phụ trong E-BDL làm cơ sở để nhà thầu lập E-HSDT
-B. Năng lực và kinh nghiệm của nhà thầu phụ sẽ không được xem xét khi đánh giá E-HSDT của nhà thầu
-C. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ trong danh sách các nhà thầu phụ nêu trong
-E-HSDT
-D. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ được chủ đầu tư chấp thuận để tham gia thực hiện cung cấp dịch vụ liên quan</t>
-  </si>
-  <si>
     <t>A. Phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó để sửa đổi cho phù hợp và tiến hành nộp lại E-HSDT mới
 B. Không phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó, chỉ cần sửa đổi cho phù hợp và tiến hành nộp lại E-HSDT mới
 C. Sửa đổi cho phù hợp E-HSDT đã nộp mà không phải nộp lại E- HSDT mới
@@ -3836,6 +3815,24 @@
 B. Hệ thống tự động xếp hạng nhà thầu theo giá dự thầu sau khi trừ đi giá trị giảm giá (nếu có) thấp nhất (không phải phê duyệt danh sách xếp hạng nhà thầu) đối với gói thầu áp dụng quy trình 02
 C. Trường hợp có từ 02 nhà thầu trở lên cùng xếp thứ nhất thì không đánh giá theo quy trình 02 mà phải đánh giá theo quy trình 01
 D. Cả 3 đáp án đều đúng</t>
+  </si>
+  <si>
+    <t>A. Cấm tham gia hoạt động đấu thầu từ 03 năm đến 05 năm đối với thành viên A
+B. Cấm tham gia hoạt động đấu thầu từ 01 năm đến dưới 03 năm đối với thành viên A
+C. Cấm tham gia hoạt động đấu thầu từ 03 năm đến 05 năm đối với tất cả thành viên trong nhà thầu liên danh A-B
+D. Cấm tham gia hoạt động đấu thầu từ 01 năm đến 03 năm đối với tất cả thành viên trong nhà thầu liên danh A-B</t>
+  </si>
+  <si>
+    <t>A. Phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó để sửa đổi cho phù hợp và tiến hành nộp lại E-HSDT mới
+B. Không phải tiến hành rút toàn bộ E-HSDT đã nộp trước đó, chỉ cần sửa đổi cho phù hợp và tiến hành nộp lại E-HSDT mới
+C. Sửa đổi cho phù hợp E-HSDT đã nộp mà không phải nộp lại E- HSDT mới
+D. Các phương án trên đều sai</t>
+  </si>
+  <si>
+    <t>A. Chủ đầu tư phải ghi tỷ lệ % giá trị dành cho nhà thầu phụ trong E-BDL làm cơ sở để nhà thầu lập E-HSDT
+B. Năng lực và kinh nghiệm của nhà thầu phụ sẽ không được xem xét khi đánh giá E-HSDT của nhà thầu
+C. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ trong danh sách các nhà thầu phụ nêu trong E-HSDT
+D. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ được chủ đầu tư chấp thuận để tham gia thực hiện cung cấp dịch vụ liên quan</t>
   </si>
 </sst>
 </file>
@@ -5726,7 +5723,7 @@
         <v>341</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D77" s="19" t="s">
         <v>1</v>
@@ -5746,7 +5743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" ht="93" x14ac:dyDescent="0.35">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -5774,7 +5771,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A81" s="7">
         <v>80</v>
       </c>
@@ -5782,7 +5779,7 @@
         <v>58</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
       <c r="D81" s="19" t="s">
         <v>1</v>
@@ -6048,13 +6045,13 @@
         <v>4</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="D100" s="26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -6062,7 +6059,7 @@
         <v>66</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>375</v>
+        <v>782</v>
       </c>
       <c r="D101" s="21" t="s">
         <v>17</v>
@@ -6073,10 +6070,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="C102" s="14" t="s">
         <v>376</v>
-      </c>
-      <c r="C102" s="14" t="s">
-        <v>377</v>
       </c>
       <c r="D102" s="22" t="s">
         <v>0</v>
@@ -6090,7 +6087,7 @@
         <v>67</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D103" s="20" t="s">
         <v>17</v>
@@ -6104,21 +6101,21 @@
         <v>68</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D104" s="24" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="93" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A105" s="10">
         <v>104</v>
       </c>
       <c r="B105" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="C105" s="14" t="s">
         <v>380</v>
-      </c>
-      <c r="C105" s="14" t="s">
-        <v>381</v>
       </c>
       <c r="D105" s="20" t="s">
         <v>17</v>
@@ -6129,10 +6126,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="C106" s="14" t="s">
         <v>382</v>
-      </c>
-      <c r="C106" s="14" t="s">
-        <v>383</v>
       </c>
       <c r="D106" s="18" t="s">
         <v>17</v>
@@ -6146,7 +6143,7 @@
         <v>69</v>
       </c>
       <c r="C107" s="14" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>20</v>
@@ -6160,7 +6157,7 @@
         <v>70</v>
       </c>
       <c r="C108" s="14" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D108" s="21" t="s">
         <v>20</v>
@@ -6174,7 +6171,7 @@
         <v>71</v>
       </c>
       <c r="C109" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D109" s="21" t="s">
         <v>20</v>
@@ -6188,7 +6185,7 @@
         <v>72</v>
       </c>
       <c r="C110" s="14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D110" s="20" t="s">
         <v>17</v>
@@ -6199,10 +6196,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C111" s="14" t="s">
         <v>387</v>
-      </c>
-      <c r="C111" s="14" t="s">
-        <v>388</v>
       </c>
       <c r="D111" s="19" t="s">
         <v>20</v>
@@ -6213,10 +6210,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="11" t="s">
+        <v>388</v>
+      </c>
+      <c r="C112" s="14" t="s">
         <v>389</v>
-      </c>
-      <c r="C112" s="14" t="s">
-        <v>390</v>
       </c>
       <c r="D112" s="19" t="s">
         <v>17</v>
@@ -6227,10 +6224,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C113" s="14" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="D113" s="19" t="s">
         <v>1</v>
@@ -6241,38 +6238,38 @@
         <v>113</v>
       </c>
       <c r="B114" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="C114" s="30" t="s">
         <v>392</v>
-      </c>
-      <c r="C114" s="30" t="s">
-        <v>393</v>
       </c>
       <c r="D114" s="15" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="62" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A115" s="28">
         <v>114</v>
       </c>
       <c r="B115" s="30" t="s">
+        <v>393</v>
+      </c>
+      <c r="C115" s="30" t="s">
         <v>394</v>
-      </c>
-      <c r="C115" s="30" t="s">
-        <v>395</v>
       </c>
       <c r="D115" s="15" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="62" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A116" s="29">
         <v>115</v>
       </c>
       <c r="B116" s="30" t="s">
+        <v>395</v>
+      </c>
+      <c r="C116" s="30" t="s">
         <v>396</v>
-      </c>
-      <c r="C116" s="30" t="s">
-        <v>397</v>
       </c>
       <c r="D116" s="12" t="s">
         <v>1</v>
@@ -6283,16 +6280,16 @@
         <v>116</v>
       </c>
       <c r="B117" s="30" t="s">
+        <v>397</v>
+      </c>
+      <c r="C117" s="30" t="s">
         <v>398</v>
-      </c>
-      <c r="C117" s="30" t="s">
-        <v>399</v>
       </c>
       <c r="D117" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="93" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A118" s="28">
         <v>117</v>
       </c>
@@ -6300,7 +6297,7 @@
         <v>73</v>
       </c>
       <c r="C118" s="30" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D118" s="12" t="s">
         <v>20</v>
@@ -6314,7 +6311,7 @@
         <v>74</v>
       </c>
       <c r="C119" s="30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D119" s="12" t="s">
         <v>0</v>
@@ -6328,7 +6325,7 @@
         <v>75</v>
       </c>
       <c r="C120" s="30" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D120" s="12" t="s">
         <v>20</v>
@@ -6339,10 +6336,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="11" t="s">
+        <v>402</v>
+      </c>
+      <c r="C121" s="14" t="s">
         <v>403</v>
-      </c>
-      <c r="C121" s="14" t="s">
-        <v>404</v>
       </c>
       <c r="D121" s="15" t="s">
         <v>1</v>
@@ -6356,7 +6353,7 @@
         <v>76</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D122" s="15" t="s">
         <v>1</v>
@@ -6370,7 +6367,7 @@
         <v>77</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D123" s="15" t="s">
         <v>1</v>
@@ -6381,10 +6378,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="D124" s="19" t="s">
         <v>0</v>
@@ -6398,7 +6395,7 @@
         <v>78</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D125" s="21" t="s">
         <v>1</v>
@@ -6409,10 +6406,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="C126" s="14" t="s">
         <v>409</v>
-      </c>
-      <c r="C126" s="14" t="s">
-        <v>410</v>
       </c>
       <c r="D126" s="21" t="s">
         <v>17</v>
@@ -6426,7 +6423,7 @@
         <v>79</v>
       </c>
       <c r="C127" s="14" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D127" s="21" t="s">
         <v>0</v>
@@ -6440,7 +6437,7 @@
         <v>80</v>
       </c>
       <c r="C128" s="14" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D128" s="19" t="s">
         <v>0</v>
@@ -6454,7 +6451,7 @@
         <v>81</v>
       </c>
       <c r="C129" s="14" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="D129" s="19" t="s">
         <v>1</v>
@@ -6468,7 +6465,7 @@
         <v>82</v>
       </c>
       <c r="C130" s="14" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D130" s="22" t="s">
         <v>1</v>
@@ -6482,7 +6479,7 @@
         <v>83</v>
       </c>
       <c r="C131" s="14" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D131" s="22" t="s">
         <v>20</v>
@@ -6496,7 +6493,7 @@
         <v>84</v>
       </c>
       <c r="C132" s="14" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D132" s="19" t="s">
         <v>1</v>
@@ -6507,10 +6504,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="C133" s="14" t="s">
         <v>417</v>
-      </c>
-      <c r="C133" s="14" t="s">
-        <v>418</v>
       </c>
       <c r="D133" s="15" t="s">
         <v>1</v>
@@ -6521,10 +6518,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="C134" s="14" t="s">
         <v>419</v>
-      </c>
-      <c r="C134" s="14" t="s">
-        <v>420</v>
       </c>
       <c r="D134" s="31" t="s">
         <v>0</v>
@@ -6538,7 +6535,7 @@
         <v>85</v>
       </c>
       <c r="C135" s="14" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D135" s="19" t="s">
         <v>20</v>
@@ -6549,10 +6546,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="C136" s="14" t="s">
         <v>422</v>
-      </c>
-      <c r="C136" s="14" t="s">
-        <v>423</v>
       </c>
       <c r="D136" s="21" t="s">
         <v>0</v>
@@ -6566,7 +6563,7 @@
         <v>86</v>
       </c>
       <c r="C137" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D137" s="24" t="s">
         <v>0</v>
@@ -6580,7 +6577,7 @@
         <v>87</v>
       </c>
       <c r="C138" s="14" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D138" s="22" t="s">
         <v>1</v>
@@ -6594,7 +6591,7 @@
         <v>88</v>
       </c>
       <c r="C139" s="14" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D139" s="22" t="s">
         <v>0</v>
@@ -6608,7 +6605,7 @@
         <v>89</v>
       </c>
       <c r="C140" s="14" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D140" s="18" t="s">
         <v>17</v>
@@ -6622,7 +6619,7 @@
         <v>90</v>
       </c>
       <c r="C141" s="14" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D141" s="20" t="s">
         <v>17</v>
@@ -6633,10 +6630,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="C142" s="14" t="s">
         <v>428</v>
-      </c>
-      <c r="C142" s="14" t="s">
-        <v>429</v>
       </c>
       <c r="D142" s="22" t="s">
         <v>1</v>
@@ -6650,7 +6647,7 @@
         <v>91</v>
       </c>
       <c r="C143" s="14" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D143" s="18" t="s">
         <v>20</v>
@@ -6664,7 +6661,7 @@
         <v>92</v>
       </c>
       <c r="C144" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D144" s="15" t="s">
         <v>17</v>
@@ -6678,7 +6675,7 @@
         <v>93</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D145" s="19" t="s">
         <v>17</v>
@@ -6689,10 +6686,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="D146" s="19" t="s">
         <v>20</v>
@@ -6703,10 +6700,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="C147" s="14" t="s">
         <v>433</v>
-      </c>
-      <c r="C147" s="14" t="s">
-        <v>434</v>
       </c>
       <c r="D147" s="24" t="s">
         <v>1</v>
@@ -6717,10 +6714,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="C148" s="14" t="s">
         <v>435</v>
-      </c>
-      <c r="C148" s="14" t="s">
-        <v>436</v>
       </c>
       <c r="D148" s="19" t="s">
         <v>17</v>
@@ -6734,7 +6731,7 @@
         <v>94</v>
       </c>
       <c r="C149" s="14" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D149" s="21" t="s">
         <v>20</v>
@@ -6745,10 +6742,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="C150" s="14" t="s">
         <v>438</v>
-      </c>
-      <c r="C150" s="14" t="s">
-        <v>439</v>
       </c>
       <c r="D150" s="24" t="s">
         <v>20</v>
@@ -6762,7 +6759,7 @@
         <v>95</v>
       </c>
       <c r="C151" s="14" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D151" s="24" t="s">
         <v>17</v>
@@ -6776,7 +6773,7 @@
         <v>96</v>
       </c>
       <c r="C152" s="14" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D152" s="22" t="s">
         <v>1</v>
@@ -6787,10 +6784,10 @@
         <v>152</v>
       </c>
       <c r="B153" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="C153" s="14" t="s">
         <v>442</v>
-      </c>
-      <c r="C153" s="14" t="s">
-        <v>443</v>
       </c>
       <c r="D153" s="18" t="s">
         <v>0</v>
@@ -6801,10 +6798,10 @@
         <v>153</v>
       </c>
       <c r="B154" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="C154" s="14" t="s">
         <v>444</v>
-      </c>
-      <c r="C154" s="14" t="s">
-        <v>445</v>
       </c>
       <c r="D154" s="18" t="s">
         <v>1</v>
@@ -6818,7 +6815,7 @@
         <v>97</v>
       </c>
       <c r="C155" s="14" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D155" s="19" t="s">
         <v>17</v>
@@ -6829,10 +6826,10 @@
         <v>155</v>
       </c>
       <c r="B156" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="C156" s="14" t="s">
         <v>447</v>
-      </c>
-      <c r="C156" s="14" t="s">
-        <v>448</v>
       </c>
       <c r="D156" s="18" t="s">
         <v>17</v>
@@ -6843,10 +6840,10 @@
         <v>156</v>
       </c>
       <c r="B157" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="C157" s="14" t="s">
         <v>449</v>
-      </c>
-      <c r="C157" s="14" t="s">
-        <v>450</v>
       </c>
       <c r="D157" s="15" t="s">
         <v>17</v>
@@ -6860,7 +6857,7 @@
         <v>98</v>
       </c>
       <c r="C158" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D158" s="18" t="s">
         <v>0</v>
@@ -6871,10 +6868,10 @@
         <v>158</v>
       </c>
       <c r="B159" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="C159" s="14" t="s">
         <v>452</v>
-      </c>
-      <c r="C159" s="14" t="s">
-        <v>453</v>
       </c>
       <c r="D159" s="18" t="s">
         <v>1</v>
@@ -6888,7 +6885,7 @@
         <v>99</v>
       </c>
       <c r="C160" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D160" s="18" t="s">
         <v>17</v>
@@ -6899,10 +6896,10 @@
         <v>160</v>
       </c>
       <c r="B161" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="C161" s="14" t="s">
         <v>455</v>
-      </c>
-      <c r="C161" s="14" t="s">
-        <v>456</v>
       </c>
       <c r="D161" s="23" t="s">
         <v>20</v>
@@ -6916,7 +6913,7 @@
         <v>100</v>
       </c>
       <c r="C162" s="14" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D162" s="18" t="s">
         <v>0</v>
@@ -6927,24 +6924,24 @@
         <v>162</v>
       </c>
       <c r="B163" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="C163" s="14" t="s">
         <v>458</v>
-      </c>
-      <c r="C163" s="14" t="s">
-        <v>459</v>
       </c>
       <c r="D163" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="164" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A164" s="10">
         <v>163</v>
       </c>
       <c r="B164" s="11" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C164" s="14" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="D164" s="24" t="s">
         <v>1</v>
@@ -6955,10 +6952,10 @@
         <v>164</v>
       </c>
       <c r="B165" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C165" s="14" t="s">
         <v>461</v>
-      </c>
-      <c r="C165" s="14" t="s">
-        <v>462</v>
       </c>
       <c r="D165" s="21" t="s">
         <v>17</v>
@@ -6969,10 +6966,10 @@
         <v>165</v>
       </c>
       <c r="B166" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="C166" s="14" t="s">
         <v>463</v>
-      </c>
-      <c r="C166" s="14" t="s">
-        <v>464</v>
       </c>
       <c r="D166" s="18" t="s">
         <v>20</v>
@@ -6983,10 +6980,10 @@
         <v>166</v>
       </c>
       <c r="B167" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="C167" s="14" t="s">
         <v>465</v>
-      </c>
-      <c r="C167" s="14" t="s">
-        <v>466</v>
       </c>
       <c r="D167" s="20" t="s">
         <v>20</v>
@@ -6997,10 +6994,10 @@
         <v>167</v>
       </c>
       <c r="B168" s="11" t="s">
+        <v>466</v>
+      </c>
+      <c r="C168" s="14" t="s">
         <v>467</v>
-      </c>
-      <c r="C168" s="14" t="s">
-        <v>468</v>
       </c>
       <c r="D168" s="18" t="s">
         <v>0</v>
@@ -7014,7 +7011,7 @@
         <v>101</v>
       </c>
       <c r="C169" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D169" s="26" t="s">
         <v>1</v>
@@ -7025,10 +7022,10 @@
         <v>169</v>
       </c>
       <c r="B170" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C170" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D170" s="21" t="s">
         <v>17</v>
@@ -7042,7 +7039,7 @@
         <v>102</v>
       </c>
       <c r="C171" s="14" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D171" s="20" t="s">
         <v>17</v>
@@ -7056,7 +7053,7 @@
         <v>103</v>
       </c>
       <c r="C172" s="14" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D172" s="19" t="s">
         <v>20</v>
@@ -7067,10 +7064,10 @@
         <v>172</v>
       </c>
       <c r="B173" s="11" t="s">
+        <v>472</v>
+      </c>
+      <c r="C173" s="14" t="s">
         <v>473</v>
-      </c>
-      <c r="C173" s="14" t="s">
-        <v>474</v>
       </c>
       <c r="D173" s="19" t="s">
         <v>1</v>
@@ -7084,7 +7081,7 @@
         <v>104</v>
       </c>
       <c r="C174" s="14" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D174" s="19" t="s">
         <v>17</v>
@@ -7095,10 +7092,10 @@
         <v>174</v>
       </c>
       <c r="B175" s="11" t="s">
+        <v>475</v>
+      </c>
+      <c r="C175" s="14" t="s">
         <v>476</v>
-      </c>
-      <c r="C175" s="14" t="s">
-        <v>477</v>
       </c>
       <c r="D175" s="19" t="s">
         <v>17</v>
@@ -7112,7 +7109,7 @@
         <v>105</v>
       </c>
       <c r="C176" s="14" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D176" s="19" t="s">
         <v>17</v>
@@ -7123,10 +7120,10 @@
         <v>176</v>
       </c>
       <c r="B177" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="C177" s="14" t="s">
         <v>479</v>
-      </c>
-      <c r="C177" s="14" t="s">
-        <v>480</v>
       </c>
       <c r="D177" s="19" t="s">
         <v>0</v>
@@ -7137,10 +7134,10 @@
         <v>177</v>
       </c>
       <c r="B178" s="11" t="s">
+        <v>480</v>
+      </c>
+      <c r="C178" s="14" t="s">
         <v>481</v>
-      </c>
-      <c r="C178" s="14" t="s">
-        <v>482</v>
       </c>
       <c r="D178" s="19" t="s">
         <v>17</v>
@@ -7151,10 +7148,10 @@
         <v>178</v>
       </c>
       <c r="B179" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="C179" s="14" t="s">
         <v>483</v>
-      </c>
-      <c r="C179" s="14" t="s">
-        <v>484</v>
       </c>
       <c r="D179" s="19" t="s">
         <v>20</v>
@@ -7165,10 +7162,10 @@
         <v>179</v>
       </c>
       <c r="B180" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="C180" s="14" t="s">
         <v>485</v>
-      </c>
-      <c r="C180" s="14" t="s">
-        <v>486</v>
       </c>
       <c r="D180" s="19" t="s">
         <v>17</v>
@@ -7179,10 +7176,10 @@
         <v>180</v>
       </c>
       <c r="B181" s="11" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C181" s="14" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D181" s="19" t="s">
         <v>0</v>
@@ -7193,10 +7190,10 @@
         <v>181</v>
       </c>
       <c r="B182" s="11" t="s">
+        <v>487</v>
+      </c>
+      <c r="C182" s="14" t="s">
         <v>488</v>
-      </c>
-      <c r="C182" s="14" t="s">
-        <v>489</v>
       </c>
       <c r="D182" s="19" t="s">
         <v>1</v>
@@ -7210,7 +7207,7 @@
         <v>106</v>
       </c>
       <c r="C183" s="14" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D183" s="19" t="s">
         <v>20</v>
@@ -7224,7 +7221,7 @@
         <v>107</v>
       </c>
       <c r="C184" s="14" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D184" s="19" t="s">
         <v>17</v>
@@ -7238,7 +7235,7 @@
         <v>108</v>
       </c>
       <c r="C185" s="14" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D185" s="19" t="s">
         <v>0</v>
@@ -7249,10 +7246,10 @@
         <v>185</v>
       </c>
       <c r="B186" s="11" t="s">
+        <v>492</v>
+      </c>
+      <c r="C186" s="14" t="s">
         <v>493</v>
-      </c>
-      <c r="C186" s="14" t="s">
-        <v>494</v>
       </c>
       <c r="D186" s="19" t="s">
         <v>17</v>
@@ -7263,10 +7260,10 @@
         <v>186</v>
       </c>
       <c r="B187" s="11" t="s">
+        <v>494</v>
+      </c>
+      <c r="C187" s="14" t="s">
         <v>495</v>
-      </c>
-      <c r="C187" s="14" t="s">
-        <v>496</v>
       </c>
       <c r="D187" s="19" t="s">
         <v>20</v>
@@ -7277,10 +7274,10 @@
         <v>187</v>
       </c>
       <c r="B188" s="11" t="s">
+        <v>496</v>
+      </c>
+      <c r="C188" s="14" t="s">
         <v>497</v>
-      </c>
-      <c r="C188" s="14" t="s">
-        <v>498</v>
       </c>
       <c r="D188" s="18" t="s">
         <v>1</v>
@@ -7294,7 +7291,7 @@
         <v>109</v>
       </c>
       <c r="C189" s="14" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D189" s="18" t="s">
         <v>20</v>
@@ -7305,10 +7302,10 @@
         <v>189</v>
       </c>
       <c r="B190" s="11" t="s">
+        <v>499</v>
+      </c>
+      <c r="C190" s="14" t="s">
         <v>500</v>
-      </c>
-      <c r="C190" s="14" t="s">
-        <v>501</v>
       </c>
       <c r="D190" s="22" t="s">
         <v>1</v>
@@ -7319,10 +7316,10 @@
         <v>190</v>
       </c>
       <c r="B191" s="11" t="s">
+        <v>501</v>
+      </c>
+      <c r="C191" s="14" t="s">
         <v>502</v>
-      </c>
-      <c r="C191" s="14" t="s">
-        <v>503</v>
       </c>
       <c r="D191" s="18" t="s">
         <v>0</v>
@@ -7333,10 +7330,10 @@
         <v>191</v>
       </c>
       <c r="B192" s="11" t="s">
+        <v>503</v>
+      </c>
+      <c r="C192" s="14" t="s">
         <v>504</v>
-      </c>
-      <c r="C192" s="14" t="s">
-        <v>505</v>
       </c>
       <c r="D192" s="18" t="s">
         <v>1</v>
@@ -7350,7 +7347,7 @@
         <v>110</v>
       </c>
       <c r="C193" s="14" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D193" s="18" t="s">
         <v>0</v>
@@ -7364,7 +7361,7 @@
         <v>111</v>
       </c>
       <c r="C194" s="14" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D194" s="15" t="s">
         <v>1</v>
@@ -7375,10 +7372,10 @@
         <v>194</v>
       </c>
       <c r="B195" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="C195" s="14" t="s">
         <v>508</v>
-      </c>
-      <c r="C195" s="14" t="s">
-        <v>509</v>
       </c>
       <c r="D195" s="19" t="s">
         <v>1</v>
@@ -7389,10 +7386,10 @@
         <v>195</v>
       </c>
       <c r="B196" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="C196" s="14" t="s">
         <v>510</v>
-      </c>
-      <c r="C196" s="14" t="s">
-        <v>511</v>
       </c>
       <c r="D196" s="20" t="s">
         <v>17</v>
@@ -7406,7 +7403,7 @@
         <v>112</v>
       </c>
       <c r="C197" s="14" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D197" s="19" t="s">
         <v>1</v>
@@ -7420,21 +7417,21 @@
         <v>113</v>
       </c>
       <c r="C198" s="14" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D198" s="18" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:4" ht="62" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A199" s="10">
         <v>198</v>
       </c>
       <c r="B199" s="11" t="s">
+        <v>513</v>
+      </c>
+      <c r="C199" s="14" t="s">
         <v>514</v>
-      </c>
-      <c r="C199" s="14" t="s">
-        <v>515</v>
       </c>
       <c r="D199" s="18" t="s">
         <v>0</v>
@@ -7445,10 +7442,10 @@
         <v>199</v>
       </c>
       <c r="B200" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="C200" s="14" t="s">
         <v>516</v>
-      </c>
-      <c r="C200" s="14" t="s">
-        <v>517</v>
       </c>
       <c r="D200" s="19" t="s">
         <v>1</v>
@@ -7459,10 +7456,10 @@
         <v>200</v>
       </c>
       <c r="B201" s="11" t="s">
+        <v>517</v>
+      </c>
+      <c r="C201" s="14" t="s">
         <v>518</v>
-      </c>
-      <c r="C201" s="14" t="s">
-        <v>519</v>
       </c>
       <c r="D201" s="24" t="s">
         <v>1</v>
@@ -7476,7 +7473,7 @@
         <v>114</v>
       </c>
       <c r="C202" s="14" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D202" s="23" t="s">
         <v>20</v>
@@ -7490,7 +7487,7 @@
         <v>115</v>
       </c>
       <c r="C203" s="14" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="D203" s="24" t="s">
         <v>17</v>
@@ -7504,21 +7501,21 @@
         <v>116</v>
       </c>
       <c r="C204" s="14" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D204" s="24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="205" spans="1:4" ht="62" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A205" s="4">
         <v>204</v>
       </c>
       <c r="B205" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="C205" s="14" t="s">
         <v>522</v>
-      </c>
-      <c r="C205" s="14" t="s">
-        <v>523</v>
       </c>
       <c r="D205" s="18" t="s">
         <v>0</v>
@@ -7529,10 +7526,10 @@
         <v>205</v>
       </c>
       <c r="B206" s="11" t="s">
+        <v>523</v>
+      </c>
+      <c r="C206" s="14" t="s">
         <v>524</v>
-      </c>
-      <c r="C206" s="14" t="s">
-        <v>525</v>
       </c>
       <c r="D206" s="18" t="s">
         <v>1</v>
@@ -7546,7 +7543,7 @@
         <v>117</v>
       </c>
       <c r="C207" s="14" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D207" s="19" t="s">
         <v>20</v>
@@ -7557,10 +7554,10 @@
         <v>207</v>
       </c>
       <c r="B208" s="11" t="s">
+        <v>526</v>
+      </c>
+      <c r="C208" s="14" t="s">
         <v>527</v>
-      </c>
-      <c r="C208" s="14" t="s">
-        <v>528</v>
       </c>
       <c r="D208" s="18" t="s">
         <v>1</v>
@@ -7571,10 +7568,10 @@
         <v>208</v>
       </c>
       <c r="B209" s="11" t="s">
+        <v>528</v>
+      </c>
+      <c r="C209" s="14" t="s">
         <v>529</v>
-      </c>
-      <c r="C209" s="14" t="s">
-        <v>530</v>
       </c>
       <c r="D209" s="18" t="s">
         <v>1</v>
@@ -7585,10 +7582,10 @@
         <v>209</v>
       </c>
       <c r="B210" s="11" t="s">
+        <v>530</v>
+      </c>
+      <c r="C210" s="14" t="s">
         <v>531</v>
-      </c>
-      <c r="C210" s="14" t="s">
-        <v>532</v>
       </c>
       <c r="D210" s="18" t="s">
         <v>0</v>
@@ -7599,10 +7596,10 @@
         <v>210</v>
       </c>
       <c r="B211" s="11" t="s">
+        <v>532</v>
+      </c>
+      <c r="C211" s="14" t="s">
         <v>533</v>
-      </c>
-      <c r="C211" s="14" t="s">
-        <v>534</v>
       </c>
       <c r="D211" s="32" t="s">
         <v>17</v>
@@ -7613,10 +7610,10 @@
         <v>211</v>
       </c>
       <c r="B212" s="11" t="s">
+        <v>534</v>
+      </c>
+      <c r="C212" s="14" t="s">
         <v>535</v>
-      </c>
-      <c r="C212" s="14" t="s">
-        <v>536</v>
       </c>
       <c r="D212" s="21" t="s">
         <v>0</v>
@@ -7627,10 +7624,10 @@
         <v>212</v>
       </c>
       <c r="B213" s="11" t="s">
+        <v>536</v>
+      </c>
+      <c r="C213" s="14" t="s">
         <v>537</v>
-      </c>
-      <c r="C213" s="14" t="s">
-        <v>538</v>
       </c>
       <c r="D213" s="32" t="s">
         <v>20</v>
@@ -7644,7 +7641,7 @@
         <v>118</v>
       </c>
       <c r="C214" s="14" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D214" s="21" t="s">
         <v>0</v>
@@ -7658,7 +7655,7 @@
         <v>119</v>
       </c>
       <c r="C215" s="14" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D215" s="15" t="s">
         <v>20</v>
@@ -7669,10 +7666,10 @@
         <v>215</v>
       </c>
       <c r="B216" s="11" t="s">
+        <v>540</v>
+      </c>
+      <c r="C216" s="14" t="s">
         <v>541</v>
-      </c>
-      <c r="C216" s="14" t="s">
-        <v>542</v>
       </c>
       <c r="D216" s="19" t="s">
         <v>20</v>
@@ -7686,7 +7683,7 @@
         <v>120</v>
       </c>
       <c r="C217" s="14" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D217" s="18" t="s">
         <v>0</v>
@@ -7700,7 +7697,7 @@
         <v>121</v>
       </c>
       <c r="C218" s="14" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D218" s="20" t="s">
         <v>20</v>
@@ -7711,10 +7708,10 @@
         <v>218</v>
       </c>
       <c r="B219" s="11" t="s">
+        <v>544</v>
+      </c>
+      <c r="C219" s="14" t="s">
         <v>545</v>
-      </c>
-      <c r="C219" s="14" t="s">
-        <v>546</v>
       </c>
       <c r="D219" s="20" t="s">
         <v>17</v>
@@ -7725,10 +7722,10 @@
         <v>219</v>
       </c>
       <c r="B220" s="11" t="s">
+        <v>546</v>
+      </c>
+      <c r="C220" s="14" t="s">
         <v>547</v>
-      </c>
-      <c r="C220" s="14" t="s">
-        <v>548</v>
       </c>
       <c r="D220" s="19" t="s">
         <v>20</v>
@@ -7742,7 +7739,7 @@
         <v>122</v>
       </c>
       <c r="C221" s="14" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D221" s="18" t="s">
         <v>17</v>
@@ -7756,7 +7753,7 @@
         <v>123</v>
       </c>
       <c r="C222" s="14" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D222" s="18" t="s">
         <v>0</v>
@@ -7770,7 +7767,7 @@
         <v>124</v>
       </c>
       <c r="C223" s="14" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D223" s="18" t="s">
         <v>0</v>
@@ -7784,7 +7781,7 @@
         <v>125</v>
       </c>
       <c r="C224" s="14" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D224" s="18" t="s">
         <v>0</v>
@@ -7798,7 +7795,7 @@
         <v>126</v>
       </c>
       <c r="C225" s="14" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="D225" s="18" t="s">
         <v>0</v>
@@ -7809,10 +7806,10 @@
         <v>225</v>
       </c>
       <c r="B226" s="11" t="s">
+        <v>553</v>
+      </c>
+      <c r="C226" s="14" t="s">
         <v>554</v>
-      </c>
-      <c r="C226" s="14" t="s">
-        <v>555</v>
       </c>
       <c r="D226" s="18" t="s">
         <v>1</v>
@@ -7826,7 +7823,7 @@
         <v>127</v>
       </c>
       <c r="C227" s="14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D227" s="20" t="s">
         <v>17</v>
@@ -7840,7 +7837,7 @@
         <v>128</v>
       </c>
       <c r="C228" s="14" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D228" s="18" t="s">
         <v>0</v>
@@ -7851,10 +7848,10 @@
         <v>228</v>
       </c>
       <c r="B229" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="C229" s="14" t="s">
         <v>558</v>
-      </c>
-      <c r="C229" s="14" t="s">
-        <v>559</v>
       </c>
       <c r="D229" s="20" t="s">
         <v>20</v>
@@ -7868,7 +7865,7 @@
         <v>129</v>
       </c>
       <c r="C230" s="14" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D230" s="20" t="s">
         <v>20</v>
@@ -7882,7 +7879,7 @@
         <v>130</v>
       </c>
       <c r="C231" s="14" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D231" s="19" t="s">
         <v>1</v>
@@ -7896,7 +7893,7 @@
         <v>131</v>
       </c>
       <c r="C232" s="14" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D232" s="19" t="s">
         <v>0</v>
@@ -7910,7 +7907,7 @@
         <v>132</v>
       </c>
       <c r="C233" s="14" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D233" s="20" t="s">
         <v>20</v>
@@ -7924,7 +7921,7 @@
         <v>133</v>
       </c>
       <c r="C234" s="14" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D234" s="18" t="s">
         <v>0</v>
@@ -7935,10 +7932,10 @@
         <v>234</v>
       </c>
       <c r="B235" s="11" t="s">
+        <v>564</v>
+      </c>
+      <c r="C235" s="14" t="s">
         <v>565</v>
-      </c>
-      <c r="C235" s="14" t="s">
-        <v>566</v>
       </c>
       <c r="D235" s="20" t="s">
         <v>17</v>
@@ -7952,7 +7949,7 @@
         <v>134</v>
       </c>
       <c r="C236" s="11" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D236" s="20" t="s">
         <v>0</v>
@@ -7963,10 +7960,10 @@
         <v>236</v>
       </c>
       <c r="B237" s="16" t="s">
+        <v>567</v>
+      </c>
+      <c r="C237" s="14" t="s">
         <v>568</v>
-      </c>
-      <c r="C237" s="14" t="s">
-        <v>569</v>
       </c>
       <c r="D237" s="20" t="s">
         <v>0</v>
@@ -7977,10 +7974,10 @@
         <v>237</v>
       </c>
       <c r="B238" s="11" t="s">
+        <v>569</v>
+      </c>
+      <c r="C238" s="14" t="s">
         <v>570</v>
-      </c>
-      <c r="C238" s="14" t="s">
-        <v>571</v>
       </c>
       <c r="D238" s="18" t="s">
         <v>20</v>
@@ -7994,7 +7991,7 @@
         <v>135</v>
       </c>
       <c r="C239" s="14" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D239" s="20" t="s">
         <v>0</v>
@@ -8005,10 +8002,10 @@
         <v>239</v>
       </c>
       <c r="B240" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C240" s="14" t="s">
         <v>573</v>
-      </c>
-      <c r="C240" s="14" t="s">
-        <v>574</v>
       </c>
       <c r="D240" s="20" t="s">
         <v>0</v>
@@ -8022,7 +8019,7 @@
         <v>136</v>
       </c>
       <c r="C241" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D241" s="21" t="s">
         <v>1</v>
@@ -8033,10 +8030,10 @@
         <v>241</v>
       </c>
       <c r="B242" s="5" t="s">
+        <v>575</v>
+      </c>
+      <c r="C242" s="14" t="s">
         <v>576</v>
-      </c>
-      <c r="C242" s="14" t="s">
-        <v>577</v>
       </c>
       <c r="D242" s="33" t="s">
         <v>0</v>
@@ -8047,10 +8044,10 @@
         <v>242</v>
       </c>
       <c r="B243" s="11" t="s">
+        <v>577</v>
+      </c>
+      <c r="C243" s="25" t="s">
         <v>578</v>
-      </c>
-      <c r="C243" s="25" t="s">
-        <v>579</v>
       </c>
       <c r="D243" s="20" t="s">
         <v>20</v>
@@ -8064,7 +8061,7 @@
         <v>137</v>
       </c>
       <c r="C244" s="14" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D244" s="18" t="s">
         <v>1</v>
@@ -8075,10 +8072,10 @@
         <v>244</v>
       </c>
       <c r="B245" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="C245" s="14" t="s">
         <v>581</v>
-      </c>
-      <c r="C245" s="14" t="s">
-        <v>582</v>
       </c>
       <c r="D245" s="18" t="s">
         <v>17</v>
@@ -8089,10 +8086,10 @@
         <v>245</v>
       </c>
       <c r="B246" s="11" t="s">
+        <v>582</v>
+      </c>
+      <c r="C246" s="14" t="s">
         <v>583</v>
-      </c>
-      <c r="C246" s="14" t="s">
-        <v>584</v>
       </c>
       <c r="D246" s="18" t="s">
         <v>17</v>
@@ -8103,10 +8100,10 @@
         <v>246</v>
       </c>
       <c r="B247" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="C247" s="14" t="s">
         <v>585</v>
-      </c>
-      <c r="C247" s="14" t="s">
-        <v>586</v>
       </c>
       <c r="D247" s="18" t="s">
         <v>1</v>
@@ -8120,7 +8117,7 @@
         <v>138</v>
       </c>
       <c r="C248" s="14" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D248" s="18" t="s">
         <v>20</v>
@@ -8131,10 +8128,10 @@
         <v>248</v>
       </c>
       <c r="B249" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="C249" s="14" t="s">
         <v>588</v>
-      </c>
-      <c r="C249" s="14" t="s">
-        <v>589</v>
       </c>
       <c r="D249" s="18" t="s">
         <v>20</v>
@@ -8148,7 +8145,7 @@
         <v>139</v>
       </c>
       <c r="C250" s="14" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D250" s="18" t="s">
         <v>0</v>
@@ -8159,10 +8156,10 @@
         <v>250</v>
       </c>
       <c r="B251" s="11" t="s">
+        <v>590</v>
+      </c>
+      <c r="C251" s="14" t="s">
         <v>591</v>
-      </c>
-      <c r="C251" s="14" t="s">
-        <v>592</v>
       </c>
       <c r="D251" s="19" t="s">
         <v>20</v>
@@ -8176,7 +8173,7 @@
         <v>140</v>
       </c>
       <c r="C252" s="14" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D252" s="20" t="s">
         <v>20</v>
@@ -8190,7 +8187,7 @@
         <v>141</v>
       </c>
       <c r="C253" s="14" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D253" s="20" t="s">
         <v>20</v>
@@ -8204,7 +8201,7 @@
         <v>142</v>
       </c>
       <c r="C254" s="14" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D254" s="20" t="s">
         <v>1</v>
@@ -8215,10 +8212,10 @@
         <v>254</v>
       </c>
       <c r="B255" s="11" t="s">
+        <v>595</v>
+      </c>
+      <c r="C255" s="14" t="s">
         <v>596</v>
-      </c>
-      <c r="C255" s="14" t="s">
-        <v>597</v>
       </c>
       <c r="D255" s="18" t="s">
         <v>20</v>
@@ -8229,10 +8226,10 @@
         <v>255</v>
       </c>
       <c r="B256" s="11" t="s">
+        <v>597</v>
+      </c>
+      <c r="C256" s="14" t="s">
         <v>598</v>
-      </c>
-      <c r="C256" s="14" t="s">
-        <v>599</v>
       </c>
       <c r="D256" s="18" t="s">
         <v>17</v>
@@ -8246,7 +8243,7 @@
         <v>143</v>
       </c>
       <c r="C257" s="14" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D257" s="19" t="s">
         <v>0</v>
@@ -8260,7 +8257,7 @@
         <v>144</v>
       </c>
       <c r="C258" s="14" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D258" s="18" t="s">
         <v>0</v>
@@ -8271,10 +8268,10 @@
         <v>258</v>
       </c>
       <c r="B259" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="C259" s="14" t="s">
         <v>602</v>
-      </c>
-      <c r="C259" s="14" t="s">
-        <v>603</v>
       </c>
       <c r="D259" s="19" t="s">
         <v>20</v>
@@ -8288,7 +8285,7 @@
         <v>145</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D260" s="20" t="s">
         <v>1</v>
@@ -8302,7 +8299,7 @@
         <v>146</v>
       </c>
       <c r="C261" s="14" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D261" s="18" t="s">
         <v>0</v>
@@ -8316,7 +8313,7 @@
         <v>147</v>
       </c>
       <c r="C262" s="14" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D262" s="19" t="s">
         <v>0</v>
@@ -8330,7 +8327,7 @@
         <v>148</v>
       </c>
       <c r="C263" s="25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D263" s="21" t="s">
         <v>0</v>
@@ -8341,10 +8338,10 @@
         <v>263</v>
       </c>
       <c r="B264" s="30" t="s">
+        <v>607</v>
+      </c>
+      <c r="C264" s="25" t="s">
         <v>608</v>
-      </c>
-      <c r="C264" s="25" t="s">
-        <v>609</v>
       </c>
       <c r="D264" s="19" t="s">
         <v>1</v>
@@ -8358,7 +8355,7 @@
         <v>149</v>
       </c>
       <c r="C265" s="25" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D265" s="18" t="s">
         <v>1</v>
@@ -8372,7 +8369,7 @@
         <v>150</v>
       </c>
       <c r="C266" s="14" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D266" s="35" t="s">
         <v>1</v>
@@ -8383,10 +8380,10 @@
         <v>266</v>
       </c>
       <c r="B267" s="11" t="s">
+        <v>611</v>
+      </c>
+      <c r="C267" s="14" t="s">
         <v>612</v>
-      </c>
-      <c r="C267" s="14" t="s">
-        <v>613</v>
       </c>
       <c r="D267" s="18" t="s">
         <v>0</v>
@@ -8397,10 +8394,10 @@
         <v>267</v>
       </c>
       <c r="B268" s="11" t="s">
+        <v>613</v>
+      </c>
+      <c r="C268" s="14" t="s">
         <v>614</v>
-      </c>
-      <c r="C268" s="14" t="s">
-        <v>615</v>
       </c>
       <c r="D268" s="18" t="s">
         <v>1</v>
@@ -8411,10 +8408,10 @@
         <v>268</v>
       </c>
       <c r="B269" s="11" t="s">
+        <v>615</v>
+      </c>
+      <c r="C269" s="14" t="s">
         <v>616</v>
-      </c>
-      <c r="C269" s="14" t="s">
-        <v>617</v>
       </c>
       <c r="D269" s="18" t="s">
         <v>1</v>
@@ -8428,7 +8425,7 @@
         <v>151</v>
       </c>
       <c r="C270" s="14" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D270" s="18" t="s">
         <v>1</v>
@@ -8442,7 +8439,7 @@
         <v>152</v>
       </c>
       <c r="C271" s="14" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D271" s="18" t="s">
         <v>0</v>
@@ -8453,10 +8450,10 @@
         <v>271</v>
       </c>
       <c r="B272" s="11" t="s">
+        <v>619</v>
+      </c>
+      <c r="C272" s="14" t="s">
         <v>620</v>
-      </c>
-      <c r="C272" s="14" t="s">
-        <v>621</v>
       </c>
       <c r="D272" s="18" t="s">
         <v>0</v>
@@ -8470,7 +8467,7 @@
         <v>153</v>
       </c>
       <c r="C273" s="14" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D273" s="15" t="s">
         <v>0</v>
@@ -8484,7 +8481,7 @@
         <v>154</v>
       </c>
       <c r="C274" s="14" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D274" s="19" t="s">
         <v>20</v>
@@ -8498,7 +8495,7 @@
         <v>155</v>
       </c>
       <c r="C275" s="14" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D275" s="18" t="s">
         <v>1</v>
@@ -8509,10 +8506,10 @@
         <v>275</v>
       </c>
       <c r="B276" s="11" t="s">
+        <v>624</v>
+      </c>
+      <c r="C276" s="14" t="s">
         <v>625</v>
-      </c>
-      <c r="C276" s="14" t="s">
-        <v>626</v>
       </c>
       <c r="D276" s="36" t="s">
         <v>0</v>
@@ -8523,10 +8520,10 @@
         <v>276</v>
       </c>
       <c r="B277" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="C277" s="14" t="s">
         <v>627</v>
-      </c>
-      <c r="C277" s="14" t="s">
-        <v>628</v>
       </c>
       <c r="D277" s="36" t="s">
         <v>20</v>
@@ -8537,24 +8534,24 @@
         <v>277</v>
       </c>
       <c r="B278" s="11" t="s">
+        <v>628</v>
+      </c>
+      <c r="C278" s="14" t="s">
         <v>629</v>
-      </c>
-      <c r="C278" s="14" t="s">
-        <v>630</v>
       </c>
       <c r="D278" s="36" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:4" ht="93" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:4" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A279" s="10">
         <v>278</v>
       </c>
       <c r="B279" s="11" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C279" s="14" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D279" s="36" t="s">
         <v>17</v>
@@ -8565,10 +8562,10 @@
         <v>279</v>
       </c>
       <c r="B280" s="11" t="s">
+        <v>631</v>
+      </c>
+      <c r="C280" s="14" t="s">
         <v>632</v>
-      </c>
-      <c r="C280" s="14" t="s">
-        <v>633</v>
       </c>
       <c r="D280" s="19" t="s">
         <v>20</v>
@@ -8582,7 +8579,7 @@
         <v>156</v>
       </c>
       <c r="C281" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D281" s="19" t="s">
         <v>20</v>
@@ -8596,7 +8593,7 @@
         <v>157</v>
       </c>
       <c r="C282" s="14" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D282" s="19" t="s">
         <v>17</v>
@@ -8610,7 +8607,7 @@
         <v>158</v>
       </c>
       <c r="C283" s="14" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D283" s="19" t="s">
         <v>20</v>
@@ -8624,7 +8621,7 @@
         <v>159</v>
       </c>
       <c r="C284" s="14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D284" s="19" t="s">
         <v>0</v>
@@ -8638,7 +8635,7 @@
         <v>160</v>
       </c>
       <c r="C285" s="14" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D285" s="19" t="s">
         <v>17</v>
@@ -8652,7 +8649,7 @@
         <v>161</v>
       </c>
       <c r="C286" s="14" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D286" s="19" t="s">
         <v>17</v>
@@ -8666,7 +8663,7 @@
         <v>162</v>
       </c>
       <c r="C287" s="14" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D287" s="19" t="s">
         <v>0</v>
@@ -8680,7 +8677,7 @@
         <v>163</v>
       </c>
       <c r="C288" s="14" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D288" s="19" t="s">
         <v>17</v>
@@ -8694,7 +8691,7 @@
         <v>164</v>
       </c>
       <c r="C289" s="25" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D289" s="19" t="s">
         <v>17</v>
@@ -8708,7 +8705,7 @@
         <v>165</v>
       </c>
       <c r="C290" s="14" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D290" s="19" t="s">
         <v>17</v>
@@ -8722,7 +8719,7 @@
         <v>166</v>
       </c>
       <c r="C291" s="14" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D291" s="19" t="s">
         <v>17</v>
@@ -8733,10 +8730,10 @@
         <v>291</v>
       </c>
       <c r="B292" s="11" t="s">
+        <v>644</v>
+      </c>
+      <c r="C292" s="14" t="s">
         <v>645</v>
-      </c>
-      <c r="C292" s="14" t="s">
-        <v>646</v>
       </c>
       <c r="D292" s="8" t="s">
         <v>17</v>
@@ -8747,10 +8744,10 @@
         <v>292</v>
       </c>
       <c r="B293" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="C293" s="14" t="s">
         <v>647</v>
-      </c>
-      <c r="C293" s="14" t="s">
-        <v>648</v>
       </c>
       <c r="D293" s="19" t="s">
         <v>17</v>
@@ -8761,10 +8758,10 @@
         <v>293</v>
       </c>
       <c r="B294" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="C294" s="14" t="s">
         <v>649</v>
-      </c>
-      <c r="C294" s="14" t="s">
-        <v>650</v>
       </c>
       <c r="D294" s="19" t="s">
         <v>20</v>
@@ -8778,7 +8775,7 @@
         <v>167</v>
       </c>
       <c r="C295" s="14" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D295" s="19" t="s">
         <v>20</v>
@@ -8792,7 +8789,7 @@
         <v>168</v>
       </c>
       <c r="C296" s="14" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D296" s="19" t="s">
         <v>20</v>
@@ -8806,7 +8803,7 @@
         <v>145</v>
       </c>
       <c r="C297" s="14" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D297" s="19" t="s">
         <v>0</v>
@@ -8820,7 +8817,7 @@
         <v>169</v>
       </c>
       <c r="C298" s="14" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D298" s="19" t="s">
         <v>1</v>
@@ -8834,7 +8831,7 @@
         <v>170</v>
       </c>
       <c r="C299" s="14" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D299" s="19" t="s">
         <v>0</v>
@@ -8845,10 +8842,10 @@
         <v>299</v>
       </c>
       <c r="B300" s="11" t="s">
+        <v>655</v>
+      </c>
+      <c r="C300" s="14" t="s">
         <v>656</v>
-      </c>
-      <c r="C300" s="14" t="s">
-        <v>657</v>
       </c>
       <c r="D300" s="19" t="s">
         <v>1</v>
@@ -8862,7 +8859,7 @@
         <v>171</v>
       </c>
       <c r="C301" s="14" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D301" s="15" t="s">
         <v>20</v>
@@ -8873,10 +8870,10 @@
         <v>301</v>
       </c>
       <c r="B302" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C302" s="14" t="s">
         <v>659</v>
-      </c>
-      <c r="C302" s="14" t="s">
-        <v>660</v>
       </c>
       <c r="D302" s="19" t="s">
         <v>0</v>
@@ -8890,7 +8887,7 @@
         <v>172</v>
       </c>
       <c r="C303" s="14" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D303" s="15" t="s">
         <v>17</v>
@@ -8904,7 +8901,7 @@
         <v>173</v>
       </c>
       <c r="C304" s="14" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="D304" s="19" t="s">
         <v>17</v>
@@ -8918,7 +8915,7 @@
         <v>174</v>
       </c>
       <c r="C305" s="14" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D305" s="19" t="s">
         <v>17</v>
@@ -8932,7 +8929,7 @@
         <v>175</v>
       </c>
       <c r="C306" s="14" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D306" s="19" t="s">
         <v>17</v>
@@ -8946,7 +8943,7 @@
         <v>176</v>
       </c>
       <c r="C307" s="14" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D307" s="15" t="s">
         <v>17</v>
@@ -8960,7 +8957,7 @@
         <v>177</v>
       </c>
       <c r="C308" s="14" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D308" s="19" t="s">
         <v>17</v>
@@ -8974,7 +8971,7 @@
         <v>178</v>
       </c>
       <c r="C309" s="14" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D309" s="19" t="s">
         <v>17</v>
@@ -8985,10 +8982,10 @@
         <v>309</v>
       </c>
       <c r="B310" s="11" t="s">
+        <v>667</v>
+      </c>
+      <c r="C310" s="14" t="s">
         <v>668</v>
-      </c>
-      <c r="C310" s="14" t="s">
-        <v>669</v>
       </c>
       <c r="D310" s="19" t="s">
         <v>17</v>
@@ -8999,10 +8996,10 @@
         <v>310</v>
       </c>
       <c r="B311" s="11" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="C311" s="14" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D311" s="19" t="s">
         <v>17</v>
@@ -9016,7 +9013,7 @@
         <v>179</v>
       </c>
       <c r="C312" s="14" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D312" s="19" t="s">
         <v>17</v>
@@ -9030,7 +9027,7 @@
         <v>180</v>
       </c>
       <c r="C313" s="14" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D313" s="19" t="s">
         <v>17</v>
@@ -9041,10 +9038,10 @@
         <v>313</v>
       </c>
       <c r="B314" s="11" t="s">
+        <v>672</v>
+      </c>
+      <c r="C314" s="14" t="s">
         <v>673</v>
-      </c>
-      <c r="C314" s="14" t="s">
-        <v>674</v>
       </c>
       <c r="D314" s="19" t="s">
         <v>17</v>
@@ -9058,7 +9055,7 @@
         <v>181</v>
       </c>
       <c r="C315" s="14" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="D315" s="19" t="s">
         <v>0</v>
@@ -9072,7 +9069,7 @@
         <v>182</v>
       </c>
       <c r="C316" s="14" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D316" s="19" t="s">
         <v>1</v>
@@ -9086,7 +9083,7 @@
         <v>183</v>
       </c>
       <c r="C317" s="14" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D317" s="18" t="s">
         <v>1</v>
@@ -9097,10 +9094,10 @@
         <v>317</v>
       </c>
       <c r="B318" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="C318" s="14" t="s">
         <v>678</v>
-      </c>
-      <c r="C318" s="14" t="s">
-        <v>679</v>
       </c>
       <c r="D318" s="20" t="s">
         <v>17</v>
@@ -9114,7 +9111,7 @@
         <v>184</v>
       </c>
       <c r="C319" s="14" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D319" s="19" t="s">
         <v>1</v>
@@ -9128,7 +9125,7 @@
         <v>185</v>
       </c>
       <c r="C320" s="14" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D320" s="19" t="s">
         <v>20</v>
@@ -9142,7 +9139,7 @@
         <v>186</v>
       </c>
       <c r="C321" s="14" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D321" s="18" t="s">
         <v>20</v>
@@ -9156,7 +9153,7 @@
         <v>187</v>
       </c>
       <c r="C322" s="14" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D322" s="23" t="s">
         <v>0</v>
@@ -9170,7 +9167,7 @@
         <v>188</v>
       </c>
       <c r="C323" s="14" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D323" s="22" t="s">
         <v>20</v>
@@ -9184,7 +9181,7 @@
         <v>189</v>
       </c>
       <c r="C324" s="14" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D324" s="22" t="s">
         <v>20</v>
@@ -9198,7 +9195,7 @@
         <v>190</v>
       </c>
       <c r="C325" s="14" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="D325" s="15" t="s">
         <v>1</v>
@@ -9212,7 +9209,7 @@
         <v>191</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="D326" s="19" t="s">
         <v>20</v>
@@ -9226,7 +9223,7 @@
         <v>192</v>
       </c>
       <c r="C327" s="14" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D327" s="19" t="s">
         <v>20</v>
@@ -9240,7 +9237,7 @@
         <v>193</v>
       </c>
       <c r="C328" s="14" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="D328" s="19" t="s">
         <v>17</v>
@@ -9251,10 +9248,10 @@
         <v>328</v>
       </c>
       <c r="B329" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="C329" s="14" t="s">
         <v>690</v>
-      </c>
-      <c r="C329" s="14" t="s">
-        <v>691</v>
       </c>
       <c r="D329" s="19" t="s">
         <v>17</v>
@@ -9265,10 +9262,10 @@
         <v>329</v>
       </c>
       <c r="B330" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="C330" s="14" t="s">
         <v>692</v>
-      </c>
-      <c r="C330" s="14" t="s">
-        <v>693</v>
       </c>
       <c r="D330" s="19" t="s">
         <v>17</v>
@@ -9282,7 +9279,7 @@
         <v>194</v>
       </c>
       <c r="C331" s="14" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D331" s="19" t="s">
         <v>0</v>
@@ -9293,10 +9290,10 @@
         <v>331</v>
       </c>
       <c r="B332" s="11" t="s">
+        <v>694</v>
+      </c>
+      <c r="C332" s="14" t="s">
         <v>695</v>
-      </c>
-      <c r="C332" s="14" t="s">
-        <v>696</v>
       </c>
       <c r="D332" s="23" t="s">
         <v>0</v>
@@ -9310,7 +9307,7 @@
         <v>5</v>
       </c>
       <c r="C333" s="14" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D333" s="19" t="s">
         <v>20</v>
@@ -9324,7 +9321,7 @@
         <v>195</v>
       </c>
       <c r="C334" s="14" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D334" s="19" t="s">
         <v>20</v>
@@ -9335,10 +9332,10 @@
         <v>334</v>
       </c>
       <c r="B335" s="11" t="s">
+        <v>698</v>
+      </c>
+      <c r="C335" s="14" t="s">
         <v>699</v>
-      </c>
-      <c r="C335" s="14" t="s">
-        <v>700</v>
       </c>
       <c r="D335" s="19" t="s">
         <v>20</v>
@@ -9349,10 +9346,10 @@
         <v>335</v>
       </c>
       <c r="B336" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="C336" s="14" t="s">
         <v>701</v>
-      </c>
-      <c r="C336" s="14" t="s">
-        <v>702</v>
       </c>
       <c r="D336" s="19" t="s">
         <v>20</v>
@@ -9366,7 +9363,7 @@
         <v>196</v>
       </c>
       <c r="C337" s="14" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D337" s="15" t="s">
         <v>20</v>
@@ -9380,7 +9377,7 @@
         <v>197</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D338" s="19" t="s">
         <v>1</v>
@@ -9394,7 +9391,7 @@
         <v>198</v>
       </c>
       <c r="C339" s="14" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D339" s="19" t="s">
         <v>17</v>
@@ -9405,10 +9402,10 @@
         <v>339</v>
       </c>
       <c r="B340" s="11" t="s">
+        <v>705</v>
+      </c>
+      <c r="C340" s="14" t="s">
         <v>706</v>
-      </c>
-      <c r="C340" s="14" t="s">
-        <v>707</v>
       </c>
       <c r="D340" s="19" t="s">
         <v>1</v>
@@ -9422,7 +9419,7 @@
         <v>199</v>
       </c>
       <c r="C341" s="14" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D341" s="19" t="s">
         <v>1</v>
@@ -9436,7 +9433,7 @@
         <v>200</v>
       </c>
       <c r="C342" s="11" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D342" s="19" t="s">
         <v>0</v>
@@ -9450,7 +9447,7 @@
         <v>201</v>
       </c>
       <c r="C343" s="11" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D343" s="19" t="s">
         <v>1</v>
@@ -9464,7 +9461,7 @@
         <v>202</v>
       </c>
       <c r="C344" s="11" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="D344" s="19" t="s">
         <v>0</v>
@@ -9478,7 +9475,7 @@
         <v>203</v>
       </c>
       <c r="C345" s="11" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D345" s="19" t="s">
         <v>17</v>
@@ -9489,10 +9486,10 @@
         <v>345</v>
       </c>
       <c r="B346" s="11" t="s">
+        <v>711</v>
+      </c>
+      <c r="C346" s="11" t="s">
         <v>712</v>
-      </c>
-      <c r="C346" s="11" t="s">
-        <v>713</v>
       </c>
       <c r="D346" s="19" t="s">
         <v>17</v>
@@ -9506,7 +9503,7 @@
         <v>204</v>
       </c>
       <c r="C347" s="11" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D347" s="19" t="s">
         <v>0</v>
@@ -9520,7 +9517,7 @@
         <v>205</v>
       </c>
       <c r="C348" s="11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D348" s="19" t="s">
         <v>0</v>
@@ -9534,7 +9531,7 @@
         <v>206</v>
       </c>
       <c r="C349" s="11" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D349" s="19" t="s">
         <v>0</v>
@@ -9548,7 +9545,7 @@
         <v>207</v>
       </c>
       <c r="C350" s="11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D350" s="15" t="s">
         <v>1</v>
@@ -9559,10 +9556,10 @@
         <v>350</v>
       </c>
       <c r="B351" s="11" t="s">
+        <v>717</v>
+      </c>
+      <c r="C351" s="11" t="s">
         <v>718</v>
-      </c>
-      <c r="C351" s="11" t="s">
-        <v>719</v>
       </c>
       <c r="D351" s="19" t="s">
         <v>1</v>
@@ -9576,7 +9573,7 @@
         <v>208</v>
       </c>
       <c r="C352" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D352" s="19" t="s">
         <v>20</v>
@@ -9590,7 +9587,7 @@
         <v>209</v>
       </c>
       <c r="C353" s="11" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="D353" s="19" t="s">
         <v>0</v>
@@ -9601,10 +9598,10 @@
         <v>353</v>
       </c>
       <c r="B354" s="11" t="s">
+        <v>721</v>
+      </c>
+      <c r="C354" s="11" t="s">
         <v>722</v>
-      </c>
-      <c r="C354" s="11" t="s">
-        <v>723</v>
       </c>
       <c r="D354" s="19" t="s">
         <v>20</v>
@@ -9618,7 +9615,7 @@
         <v>210</v>
       </c>
       <c r="C355" s="11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="D355" s="19" t="s">
         <v>0</v>
@@ -9629,10 +9626,10 @@
         <v>355</v>
       </c>
       <c r="B356" s="11" t="s">
+        <v>724</v>
+      </c>
+      <c r="C356" s="11" t="s">
         <v>725</v>
-      </c>
-      <c r="C356" s="11" t="s">
-        <v>726</v>
       </c>
       <c r="D356" s="19" t="s">
         <v>1</v>
@@ -9646,7 +9643,7 @@
         <v>211</v>
       </c>
       <c r="C357" s="11" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D357" s="15" t="s">
         <v>20</v>
@@ -9660,7 +9657,7 @@
         <v>6</v>
       </c>
       <c r="C358" s="11" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D358" s="34" t="s">
         <v>17</v>
@@ -9674,7 +9671,7 @@
         <v>7</v>
       </c>
       <c r="C359" s="30" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D359" s="30" t="s">
         <v>20</v>
@@ -9685,10 +9682,10 @@
         <v>359</v>
       </c>
       <c r="B360" s="11" t="s">
+        <v>729</v>
+      </c>
+      <c r="C360" s="11" t="s">
         <v>730</v>
-      </c>
-      <c r="C360" s="11" t="s">
-        <v>731</v>
       </c>
       <c r="D360" s="19" t="s">
         <v>17</v>
@@ -9699,10 +9696,10 @@
         <v>360</v>
       </c>
       <c r="B361" s="30" t="s">
+        <v>731</v>
+      </c>
+      <c r="C361" s="30" t="s">
         <v>732</v>
-      </c>
-      <c r="C361" s="30" t="s">
-        <v>733</v>
       </c>
       <c r="D361" s="15" t="s">
         <v>20</v>
@@ -9713,10 +9710,10 @@
         <v>361</v>
       </c>
       <c r="B362" s="30" t="s">
+        <v>733</v>
+      </c>
+      <c r="C362" s="30" t="s">
         <v>734</v>
-      </c>
-      <c r="C362" s="30" t="s">
-        <v>735</v>
       </c>
       <c r="D362" s="15" t="s">
         <v>17</v>
@@ -9730,7 +9727,7 @@
         <v>212</v>
       </c>
       <c r="C363" s="30" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D363" s="15" t="s">
         <v>20</v>
@@ -9744,7 +9741,7 @@
         <v>213</v>
       </c>
       <c r="C364" s="30" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D364" s="15" t="s">
         <v>0</v>
@@ -9758,7 +9755,7 @@
         <v>214</v>
       </c>
       <c r="C365" s="30" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D365" s="15" t="s">
         <v>0</v>
@@ -9772,7 +9769,7 @@
         <v>215</v>
       </c>
       <c r="C366" s="30" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D366" s="15" t="s">
         <v>20</v>
@@ -9786,7 +9783,7 @@
         <v>216</v>
       </c>
       <c r="C367" s="30" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="D367" s="15" t="s">
         <v>20</v>
@@ -9797,10 +9794,10 @@
         <v>367</v>
       </c>
       <c r="B368" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="C368" s="30" t="s">
         <v>741</v>
-      </c>
-      <c r="C368" s="30" t="s">
-        <v>742</v>
       </c>
       <c r="D368" s="15" t="s">
         <v>0</v>
@@ -9814,21 +9811,21 @@
         <v>217</v>
       </c>
       <c r="C369" s="30" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D369" s="15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="370" spans="1:4" ht="62" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A370" s="10">
         <v>369</v>
       </c>
       <c r="B370" s="30" t="s">
+        <v>743</v>
+      </c>
+      <c r="C370" s="30" t="s">
         <v>744</v>
-      </c>
-      <c r="C370" s="30" t="s">
-        <v>745</v>
       </c>
       <c r="D370" s="15" t="s">
         <v>17</v>
@@ -9842,7 +9839,7 @@
         <v>8</v>
       </c>
       <c r="C371" s="30" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D371" s="15" t="s">
         <v>1</v>
@@ -9856,7 +9853,7 @@
         <v>218</v>
       </c>
       <c r="C372" s="30" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D372" s="15" t="s">
         <v>0</v>
@@ -9870,7 +9867,7 @@
         <v>219</v>
       </c>
       <c r="C373" s="30" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D373" s="15" t="s">
         <v>1</v>
@@ -9884,7 +9881,7 @@
         <v>220</v>
       </c>
       <c r="C374" s="30" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D374" s="15" t="s">
         <v>0</v>
@@ -9898,7 +9895,7 @@
         <v>221</v>
       </c>
       <c r="C375" s="30" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="D375" s="15" t="s">
         <v>1</v>
@@ -9909,10 +9906,10 @@
         <v>375</v>
       </c>
       <c r="B376" s="11" t="s">
+        <v>750</v>
+      </c>
+      <c r="C376" s="30" t="s">
         <v>751</v>
-      </c>
-      <c r="C376" s="30" t="s">
-        <v>752</v>
       </c>
       <c r="D376" s="15" t="s">
         <v>0</v>
@@ -9926,7 +9923,7 @@
         <v>222</v>
       </c>
       <c r="C377" s="30" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="D377" s="15" t="s">
         <v>20</v>
@@ -9940,7 +9937,7 @@
         <v>223</v>
       </c>
       <c r="C378" s="30" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="D378" s="15" t="s">
         <v>17</v>
@@ -9954,7 +9951,7 @@
         <v>224</v>
       </c>
       <c r="C379" s="30" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D379" s="15" t="s">
         <v>20</v>
@@ -9968,21 +9965,21 @@
         <v>9</v>
       </c>
       <c r="C380" s="30" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D380" s="15" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="381" spans="1:4" ht="124" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:4" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A381" s="10">
         <v>380</v>
       </c>
       <c r="B381" s="30" t="s">
+        <v>756</v>
+      </c>
+      <c r="C381" s="30" t="s">
         <v>757</v>
-      </c>
-      <c r="C381" s="30" t="s">
-        <v>758</v>
       </c>
       <c r="D381" s="15" t="s">
         <v>17</v>
@@ -9996,7 +9993,7 @@
         <v>225</v>
       </c>
       <c r="C382" s="30" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D382" s="15" t="s">
         <v>1</v>
@@ -10010,7 +10007,7 @@
         <v>226</v>
       </c>
       <c r="C383" s="30" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D383" s="15" t="s">
         <v>0</v>
@@ -10024,7 +10021,7 @@
         <v>227</v>
       </c>
       <c r="C384" s="30" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D384" s="15" t="s">
         <v>0</v>
@@ -10038,7 +10035,7 @@
         <v>228</v>
       </c>
       <c r="C385" s="30" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D385" s="15" t="s">
         <v>1</v>
@@ -10052,7 +10049,7 @@
         <v>229</v>
       </c>
       <c r="C386" s="11" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D386" s="15" t="s">
         <v>17</v>
@@ -10066,7 +10063,7 @@
         <v>230</v>
       </c>
       <c r="C387" s="11" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D387" s="15" t="s">
         <v>20</v>
@@ -10080,7 +10077,7 @@
         <v>231</v>
       </c>
       <c r="C388" s="11" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D388" s="15" t="s">
         <v>17</v>
@@ -10091,10 +10088,10 @@
         <v>388</v>
       </c>
       <c r="B389" s="11" t="s">
+        <v>765</v>
+      </c>
+      <c r="C389" s="11" t="s">
         <v>766</v>
-      </c>
-      <c r="C389" s="11" t="s">
-        <v>767</v>
       </c>
       <c r="D389" s="19" t="s">
         <v>1</v>
@@ -10105,10 +10102,10 @@
         <v>389</v>
       </c>
       <c r="B390" s="11" t="s">
+        <v>767</v>
+      </c>
+      <c r="C390" s="11" t="s">
         <v>768</v>
-      </c>
-      <c r="C390" s="11" t="s">
-        <v>769</v>
       </c>
       <c r="D390" s="19" t="s">
         <v>1</v>
@@ -10122,7 +10119,7 @@
         <v>232</v>
       </c>
       <c r="C391" s="11" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D391" s="19" t="s">
         <v>1</v>
@@ -10135,11 +10132,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="6227360e-e60f-4595-9753-ac508485ddd6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10370,27 +10368,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="6227360e-e60f-4595-9753-ac508485ddd6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BC35CC7-6F58-4296-A78C-C761A4406030}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8A0EA2E-6E25-4712-9DB6-6E8798AE1CF1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="6227360e-e60f-4595-9753-ac508485ddd6"/>
-    <ds:schemaRef ds:uri="bc054b22-9395-4512-bde7-19a23f2dcff6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10415,9 +10403,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8A0EA2E-6E25-4712-9DB6-6E8798AE1CF1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BC35CC7-6F58-4296-A78C-C761A4406030}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="6227360e-e60f-4595-9753-ac508485ddd6"/>
+    <ds:schemaRef ds:uri="bc054b22-9395-4512-bde7-19a23f2dcff6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore: refresh question bank workbook
</commit_message>
<xml_diff>
--- a/data/Ngan-Hang-Cau-Hoi.xlsx
+++ b/data/Ngan-Hang-Cau-Hoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f54d0bdb7235122/Documents/My App/trac-nghiem-luat-dau-thau/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9945B2BA-DA03-453F-91C4-0EF789E4D547}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6669B6E6-5ED4-4F8F-B91B-022AC5ED8FA7}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0822E189-CD53-41B9-B216-EFA7EF505EBC}"/>
   </bookViews>
@@ -1523,13 +1523,6 @@
 không đề xuất cụ thể ký mã hiệu, nhãn hiệu, xuất xứ, hãng sản xuất thì xử lý như thế nào?</t>
   </si>
   <si>
-    <t>A. Chủ đầu tư yêu cầu nhà thầu làm rõ các thông tin này để làm cơ sở đánh giá trên cơ sở không được thay đổi giá dự thầu
-B. Tổ chuyên gia căn cứ theo cataloge, đề xuất kỹ thuật kèm theo để làm cơ sở đánh giá
-C. Hồ sơ dự thầu của nhà thầu không được xem xét, đánh giá
-D. Tiếp tục đánh giá hồ sơ dự thầu, trường hơp nhà thầu trúng thầu thì yêu cầu nhà thầu bổ sung, làm
-rõ các thông tin này</t>
-  </si>
-  <si>
     <t>A. Đánh giá năng lực, kinh nghiệm của nhà thầu phụ căn cứ theo phần công việc nhà thầu phụ đảm nhận, nhà thầu tham dự thầu không phải đáp ứng về năng lực, kinh nghiệm đối với phần công việc mà nhà thầu phụ đảm nhận
 B. Không đánh giá năng lực, kinh nghiệm của nhà thầu phụ, nhà thầu tham dự thầu vẫn phải đáp ứng về năng lực, kinh nghiệm đối với phần công việc mà nhà thầu phụ đảm nhận
 C. Do chủ đầu tư quyết định đánh giá hoặc không đánh giá năng lực, kinh nghiệm nhà thầu phụ
@@ -1714,13 +1707,6 @@
 đây?</t>
   </si>
   <si>
-    <t>A. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 24 giờ kể từ thời điểm mở thầu
-B. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 02 giờ kể từ thời điểm mở thầu
-C. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 04 giờ kể từ thời điểm mở thầu
-D. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 03 ngày làm việc kể từ thời
-điểm mở thầu</t>
-  </si>
-  <si>
     <t>Chủ đầu tư A và nhà thầu B đã ký kết hợp đồng cung cấp 11000 đơn vị hàng hóa, loại hợp đồng theo đơn giá cố định. Trong quá trình thực hiện hợp đồng, nhu cầu sử dụng thực tế mà nhà thầu phải cung cấp cho chủ đầu tư chỉ là 10500 đơn vị hàng hóa.  Hãy lựa chọn phương án đúng về sửa đổi hợp
 đồng trong trường hợp này?</t>
   </si>
@@ -1729,13 +1715,6 @@
 B. Chủ đầu tư A và nhà thầu B không cần thực hiện thủ tục sửa đổi hợp đồng, không phải ký kết văn bản sửa đổi hợp đồng
 C. Chủ đầu tư A và nhà thầu B bắt buộc phải thực hiện thủ tục ký phụ lục hợp đồng để điều chỉnh khối lượng
 D. Phương án A và C đều đúng</t>
-  </si>
-  <si>
-    <t>A. Khi có sự thay đổi về chính sách, pháp luật làm ảnh hưởng trực tiếp đến việc thực hiện hợp đồng
-B. Khi có sự kiện bất khả kháng
-C. Khi thay đổi phương thức vận chuyển, địa điểm giao hàng, dịch vụ liên quan đối với gói thầu mua sắm hàng hóa
-D. Tăng, giảm thời gian đối với hợp đồng theo thời gian; tăng, giảm chi phí trực tiếp thực hiện đối với hợp đồng chi phí cộng phí; tăng, giảm giá trị cơ sở để tính phần trăm chi phí đối với hợp đồng theo tỷ lệ phần trăm; tăng, giảm mức giảm trừ thanh toán, mức tăng giá trị thanh toán đối với hợp
-đồng theo kết quả đầu ra</t>
   </si>
   <si>
     <t xml:space="preserve">A. Hồ sơ mời quan tâm, hồ sơ mời sơ tuyển, hồ sơ mời thầu được phát hành sau 01 ngày kể từ khi thông báo mời quan tâm, thông báo mời sơ tuyển, thông báo mời thầu được đăng tải thành công trên Hệ thống mạng đấu thầu quốc gia
@@ -3833,6 +3812,24 @@
 B. Năng lực và kinh nghiệm của nhà thầu phụ sẽ không được xem xét khi đánh giá E-HSDT của nhà thầu
 C. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ trong danh sách các nhà thầu phụ nêu trong E-HSDT
 D. Nhà thầu được ký kết hợp đồng với các nhà thầu phụ được chủ đầu tư chấp thuận để tham gia thực hiện cung cấp dịch vụ liên quan</t>
+  </si>
+  <si>
+    <t>A. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 24 giờ kể từ thời điểm mở thầu
+B. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 02 giờ kể từ thời điểm mở thầu
+C. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 04 giờ kể từ thời điểm mở thầu
+D. Được đăng tải trên Hệ thống mạng đấu thầu quốc gia trong thời hạn 03 ngày làm việc kể từ thời điểm mở thầu</t>
+  </si>
+  <si>
+    <t>A. Khi có sự thay đổi về chính sách, pháp luật làm ảnh hưởng trực tiếp đến việc thực hiện hợp đồng
+B. Khi có sự kiện bất khả kháng
+C. Khi thay đổi phương thức vận chuyển, địa điểm giao hàng, dịch vụ liên quan đối với gói thầu mua sắm hàng hóa
+D. Tăng, giảm thời gian đối với hợp đồng theo thời gian; tăng, giảm chi phí trực tiếp thực hiện đối với hợp đồng chi phí cộng phí; tăng, giảm giá trị cơ sở để tính phần trăm chi phí đối với hợp đồng theo tỷ lệ phần trăm; tăng, giảm mức giảm trừ thanh toán, mức tăng giá trị thanh toán đối với hợp đồng theo kết quả đầu ra</t>
+  </si>
+  <si>
+    <t>A. Chủ đầu tư yêu cầu nhà thầu làm rõ các thông tin này để làm cơ sở đánh giá trên cơ sở không được thay đổi giá dự thầu
+B. Tổ chuyên gia căn cứ theo cataloge, đề xuất kỹ thuật kèm theo để làm cơ sở đánh giá
+C. Hồ sơ dự thầu của nhà thầu không được xem xét, đánh giá
+D. Tiếp tục đánh giá hồ sơ dự thầu, trường hơp nhà thầu trúng thầu thì yêu cầu nhà thầu bổ sung, làm rõ các thông tin này</t>
   </si>
 </sst>
 </file>
@@ -5723,7 +5720,7 @@
         <v>341</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="D77" s="19" t="s">
         <v>1</v>
@@ -5779,7 +5776,7 @@
         <v>58</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="D81" s="19" t="s">
         <v>1</v>
@@ -6009,7 +6006,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A98" s="10">
         <v>97</v>
       </c>
@@ -6017,7 +6014,7 @@
         <v>372</v>
       </c>
       <c r="C98" s="25" t="s">
-        <v>373</v>
+        <v>783</v>
       </c>
       <c r="D98" s="20" t="s">
         <v>20</v>
@@ -6031,7 +6028,7 @@
         <v>65</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D99" s="19" t="s">
         <v>17</v>
@@ -6045,7 +6042,7 @@
         <v>4</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="D100" s="26" t="s">
         <v>1</v>
@@ -6059,7 +6056,7 @@
         <v>66</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="D101" s="21" t="s">
         <v>17</v>
@@ -6070,10 +6067,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="11" t="s">
+        <v>374</v>
+      </c>
+      <c r="C102" s="14" t="s">
         <v>375</v>
-      </c>
-      <c r="C102" s="14" t="s">
-        <v>376</v>
       </c>
       <c r="D102" s="22" t="s">
         <v>0</v>
@@ -6087,7 +6084,7 @@
         <v>67</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D103" s="20" t="s">
         <v>17</v>
@@ -6101,7 +6098,7 @@
         <v>68</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D104" s="24" t="s">
         <v>1</v>
@@ -6112,10 +6109,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="11" t="s">
+        <v>378</v>
+      </c>
+      <c r="C105" s="14" t="s">
         <v>379</v>
-      </c>
-      <c r="C105" s="14" t="s">
-        <v>380</v>
       </c>
       <c r="D105" s="20" t="s">
         <v>17</v>
@@ -6126,10 +6123,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="11" t="s">
+        <v>380</v>
+      </c>
+      <c r="C106" s="14" t="s">
         <v>381</v>
-      </c>
-      <c r="C106" s="14" t="s">
-        <v>382</v>
       </c>
       <c r="D106" s="18" t="s">
         <v>17</v>
@@ -6143,7 +6140,7 @@
         <v>69</v>
       </c>
       <c r="C107" s="14" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>20</v>
@@ -6157,7 +6154,7 @@
         <v>70</v>
       </c>
       <c r="C108" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D108" s="21" t="s">
         <v>20</v>
@@ -6171,7 +6168,7 @@
         <v>71</v>
       </c>
       <c r="C109" s="14" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D109" s="21" t="s">
         <v>20</v>
@@ -6185,7 +6182,7 @@
         <v>72</v>
       </c>
       <c r="C110" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D110" s="20" t="s">
         <v>17</v>
@@ -6196,10 +6193,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="11" t="s">
+        <v>385</v>
+      </c>
+      <c r="C111" s="14" t="s">
         <v>386</v>
-      </c>
-      <c r="C111" s="14" t="s">
-        <v>387</v>
       </c>
       <c r="D111" s="19" t="s">
         <v>20</v>
@@ -6210,10 +6207,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="11" t="s">
+        <v>387</v>
+      </c>
+      <c r="C112" s="14" t="s">
         <v>388</v>
-      </c>
-      <c r="C112" s="14" t="s">
-        <v>389</v>
       </c>
       <c r="D112" s="19" t="s">
         <v>17</v>
@@ -6224,10 +6221,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C113" s="14" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="D113" s="19" t="s">
         <v>1</v>
@@ -6238,10 +6235,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="30" t="s">
+        <v>390</v>
+      </c>
+      <c r="C114" s="30" t="s">
         <v>391</v>
-      </c>
-      <c r="C114" s="30" t="s">
-        <v>392</v>
       </c>
       <c r="D114" s="15" t="s">
         <v>0</v>
@@ -6252,10 +6249,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="C115" s="30" t="s">
         <v>393</v>
-      </c>
-      <c r="C115" s="30" t="s">
-        <v>394</v>
       </c>
       <c r="D115" s="15" t="s">
         <v>1</v>
@@ -6266,10 +6263,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="30" t="s">
+        <v>394</v>
+      </c>
+      <c r="C116" s="30" t="s">
         <v>395</v>
-      </c>
-      <c r="C116" s="30" t="s">
-        <v>396</v>
       </c>
       <c r="D116" s="12" t="s">
         <v>1</v>
@@ -6280,10 +6277,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="30" t="s">
+        <v>396</v>
+      </c>
+      <c r="C117" s="30" t="s">
         <v>397</v>
-      </c>
-      <c r="C117" s="30" t="s">
-        <v>398</v>
       </c>
       <c r="D117" s="12" t="s">
         <v>1</v>
@@ -6297,7 +6294,7 @@
         <v>73</v>
       </c>
       <c r="C118" s="30" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D118" s="12" t="s">
         <v>20</v>
@@ -6311,7 +6308,7 @@
         <v>74</v>
       </c>
       <c r="C119" s="30" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D119" s="12" t="s">
         <v>0</v>
@@ -6325,7 +6322,7 @@
         <v>75</v>
       </c>
       <c r="C120" s="30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D120" s="12" t="s">
         <v>20</v>
@@ -6336,10 +6333,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="C121" s="14" t="s">
         <v>402</v>
-      </c>
-      <c r="C121" s="14" t="s">
-        <v>403</v>
       </c>
       <c r="D121" s="15" t="s">
         <v>1</v>
@@ -6353,7 +6350,7 @@
         <v>76</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D122" s="15" t="s">
         <v>1</v>
@@ -6367,7 +6364,7 @@
         <v>77</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D123" s="15" t="s">
         <v>1</v>
@@ -6378,16 +6375,16 @@
         <v>123</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="D124" s="19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A125" s="7">
         <v>124</v>
       </c>
@@ -6395,7 +6392,7 @@
         <v>78</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>407</v>
+        <v>781</v>
       </c>
       <c r="D125" s="21" t="s">
         <v>1</v>
@@ -6406,16 +6403,16 @@
         <v>125</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C126" s="14" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D126" s="21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A127" s="7">
         <v>126</v>
       </c>
@@ -6423,7 +6420,7 @@
         <v>79</v>
       </c>
       <c r="C127" s="14" t="s">
-        <v>410</v>
+        <v>782</v>
       </c>
       <c r="D127" s="21" t="s">
         <v>0</v>
@@ -6437,7 +6434,7 @@
         <v>80</v>
       </c>
       <c r="C128" s="14" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D128" s="19" t="s">
         <v>0</v>
@@ -6451,7 +6448,7 @@
         <v>81</v>
       </c>
       <c r="C129" s="14" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D129" s="19" t="s">
         <v>1</v>
@@ -6465,7 +6462,7 @@
         <v>82</v>
       </c>
       <c r="C130" s="14" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="D130" s="22" t="s">
         <v>1</v>
@@ -6479,7 +6476,7 @@
         <v>83</v>
       </c>
       <c r="C131" s="14" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D131" s="22" t="s">
         <v>20</v>
@@ -6493,7 +6490,7 @@
         <v>84</v>
       </c>
       <c r="C132" s="14" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="D132" s="19" t="s">
         <v>1</v>
@@ -6504,10 +6501,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C133" s="14" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D133" s="15" t="s">
         <v>1</v>
@@ -6518,10 +6515,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C134" s="14" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D134" s="31" t="s">
         <v>0</v>
@@ -6535,7 +6532,7 @@
         <v>85</v>
       </c>
       <c r="C135" s="14" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D135" s="19" t="s">
         <v>20</v>
@@ -6546,10 +6543,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C136" s="14" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D136" s="21" t="s">
         <v>0</v>
@@ -6563,7 +6560,7 @@
         <v>86</v>
       </c>
       <c r="C137" s="14" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D137" s="24" t="s">
         <v>0</v>
@@ -6577,7 +6574,7 @@
         <v>87</v>
       </c>
       <c r="C138" s="14" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="D138" s="22" t="s">
         <v>1</v>
@@ -6591,7 +6588,7 @@
         <v>88</v>
       </c>
       <c r="C139" s="14" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D139" s="22" t="s">
         <v>0</v>
@@ -6605,7 +6602,7 @@
         <v>89</v>
       </c>
       <c r="C140" s="14" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="D140" s="18" t="s">
         <v>17</v>
@@ -6619,7 +6616,7 @@
         <v>90</v>
       </c>
       <c r="C141" s="14" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D141" s="20" t="s">
         <v>17</v>
@@ -6630,10 +6627,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="11" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C142" s="14" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="D142" s="22" t="s">
         <v>1</v>
@@ -6647,7 +6644,7 @@
         <v>91</v>
       </c>
       <c r="C143" s="14" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="D143" s="18" t="s">
         <v>20</v>
@@ -6661,7 +6658,7 @@
         <v>92</v>
       </c>
       <c r="C144" s="14" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="D144" s="15" t="s">
         <v>17</v>
@@ -6675,7 +6672,7 @@
         <v>93</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="D145" s="19" t="s">
         <v>17</v>
@@ -6686,10 +6683,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="11" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="D146" s="19" t="s">
         <v>20</v>
@@ -6700,10 +6697,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="11" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C147" s="14" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="D147" s="24" t="s">
         <v>1</v>
@@ -6714,10 +6711,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="11" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="C148" s="14" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="D148" s="19" t="s">
         <v>17</v>
@@ -6731,7 +6728,7 @@
         <v>94</v>
       </c>
       <c r="C149" s="14" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D149" s="21" t="s">
         <v>20</v>
@@ -6742,10 +6739,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="11" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C150" s="14" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="D150" s="24" t="s">
         <v>20</v>
@@ -6759,7 +6756,7 @@
         <v>95</v>
       </c>
       <c r="C151" s="14" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D151" s="24" t="s">
         <v>17</v>
@@ -6773,7 +6770,7 @@
         <v>96</v>
       </c>
       <c r="C152" s="14" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="D152" s="22" t="s">
         <v>1</v>
@@ -6784,10 +6781,10 @@
         <v>152</v>
       </c>
       <c r="B153" s="11" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C153" s="14" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="D153" s="18" t="s">
         <v>0</v>
@@ -6798,10 +6795,10 @@
         <v>153</v>
       </c>
       <c r="B154" s="11" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C154" s="14" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="D154" s="18" t="s">
         <v>1</v>
@@ -6815,7 +6812,7 @@
         <v>97</v>
       </c>
       <c r="C155" s="14" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="D155" s="19" t="s">
         <v>17</v>
@@ -6826,10 +6823,10 @@
         <v>155</v>
       </c>
       <c r="B156" s="11" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C156" s="14" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="D156" s="18" t="s">
         <v>17</v>
@@ -6840,10 +6837,10 @@
         <v>156</v>
       </c>
       <c r="B157" s="11" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="C157" s="14" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D157" s="15" t="s">
         <v>17</v>
@@ -6857,7 +6854,7 @@
         <v>98</v>
       </c>
       <c r="C158" s="14" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="D158" s="18" t="s">
         <v>0</v>
@@ -6868,10 +6865,10 @@
         <v>158</v>
       </c>
       <c r="B159" s="11" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="C159" s="14" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D159" s="18" t="s">
         <v>1</v>
@@ -6885,7 +6882,7 @@
         <v>99</v>
       </c>
       <c r="C160" s="14" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="D160" s="18" t="s">
         <v>17</v>
@@ -6896,10 +6893,10 @@
         <v>160</v>
       </c>
       <c r="B161" s="11" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C161" s="14" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="D161" s="23" t="s">
         <v>20</v>
@@ -6913,7 +6910,7 @@
         <v>100</v>
       </c>
       <c r="C162" s="14" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D162" s="18" t="s">
         <v>0</v>
@@ -6924,10 +6921,10 @@
         <v>162</v>
       </c>
       <c r="B163" s="11" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C163" s="14" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="D163" s="18" t="s">
         <v>20</v>
@@ -6938,10 +6935,10 @@
         <v>163</v>
       </c>
       <c r="B164" s="11" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="C164" s="14" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="D164" s="24" t="s">
         <v>1</v>
@@ -6952,10 +6949,10 @@
         <v>164</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="C165" s="14" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="D165" s="21" t="s">
         <v>17</v>
@@ -6966,10 +6963,10 @@
         <v>165</v>
       </c>
       <c r="B166" s="11" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C166" s="14" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="D166" s="18" t="s">
         <v>20</v>
@@ -6980,10 +6977,10 @@
         <v>166</v>
       </c>
       <c r="B167" s="11" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="C167" s="14" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="D167" s="20" t="s">
         <v>20</v>
@@ -6994,10 +6991,10 @@
         <v>167</v>
       </c>
       <c r="B168" s="11" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C168" s="14" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="D168" s="18" t="s">
         <v>0</v>
@@ -7011,7 +7008,7 @@
         <v>101</v>
       </c>
       <c r="C169" s="14" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D169" s="26" t="s">
         <v>1</v>
@@ -7022,10 +7019,10 @@
         <v>169</v>
       </c>
       <c r="B170" s="11" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C170" s="14" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D170" s="21" t="s">
         <v>17</v>
@@ -7039,7 +7036,7 @@
         <v>102</v>
       </c>
       <c r="C171" s="14" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D171" s="20" t="s">
         <v>17</v>
@@ -7053,7 +7050,7 @@
         <v>103</v>
       </c>
       <c r="C172" s="14" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="D172" s="19" t="s">
         <v>20</v>
@@ -7064,10 +7061,10 @@
         <v>172</v>
       </c>
       <c r="B173" s="11" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="D173" s="19" t="s">
         <v>1</v>
@@ -7081,7 +7078,7 @@
         <v>104</v>
       </c>
       <c r="C174" s="14" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="D174" s="19" t="s">
         <v>17</v>
@@ -7092,10 +7089,10 @@
         <v>174</v>
       </c>
       <c r="B175" s="11" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="C175" s="14" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="D175" s="19" t="s">
         <v>17</v>
@@ -7109,7 +7106,7 @@
         <v>105</v>
       </c>
       <c r="C176" s="14" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="D176" s="19" t="s">
         <v>17</v>
@@ -7120,10 +7117,10 @@
         <v>176</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="C177" s="14" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="D177" s="19" t="s">
         <v>0</v>
@@ -7134,10 +7131,10 @@
         <v>177</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="C178" s="14" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="D178" s="19" t="s">
         <v>17</v>
@@ -7148,10 +7145,10 @@
         <v>178</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="C179" s="14" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="D179" s="19" t="s">
         <v>20</v>
@@ -7162,10 +7159,10 @@
         <v>179</v>
       </c>
       <c r="B180" s="11" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C180" s="14" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D180" s="19" t="s">
         <v>17</v>
@@ -7176,10 +7173,10 @@
         <v>180</v>
       </c>
       <c r="B181" s="11" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="C181" s="14" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D181" s="19" t="s">
         <v>0</v>
@@ -7190,10 +7187,10 @@
         <v>181</v>
       </c>
       <c r="B182" s="11" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C182" s="14" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D182" s="19" t="s">
         <v>1</v>
@@ -7207,7 +7204,7 @@
         <v>106</v>
       </c>
       <c r="C183" s="14" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="D183" s="19" t="s">
         <v>20</v>
@@ -7221,7 +7218,7 @@
         <v>107</v>
       </c>
       <c r="C184" s="14" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="D184" s="19" t="s">
         <v>17</v>
@@ -7235,7 +7232,7 @@
         <v>108</v>
       </c>
       <c r="C185" s="14" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D185" s="19" t="s">
         <v>0</v>
@@ -7246,10 +7243,10 @@
         <v>185</v>
       </c>
       <c r="B186" s="11" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C186" s="14" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D186" s="19" t="s">
         <v>17</v>
@@ -7260,10 +7257,10 @@
         <v>186</v>
       </c>
       <c r="B187" s="11" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C187" s="14" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="D187" s="19" t="s">
         <v>20</v>
@@ -7274,10 +7271,10 @@
         <v>187</v>
       </c>
       <c r="B188" s="11" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C188" s="14" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D188" s="18" t="s">
         <v>1</v>
@@ -7291,7 +7288,7 @@
         <v>109</v>
       </c>
       <c r="C189" s="14" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="D189" s="18" t="s">
         <v>20</v>
@@ -7302,10 +7299,10 @@
         <v>189</v>
       </c>
       <c r="B190" s="11" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C190" s="14" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D190" s="22" t="s">
         <v>1</v>
@@ -7316,10 +7313,10 @@
         <v>190</v>
       </c>
       <c r="B191" s="11" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="C191" s="14" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="D191" s="18" t="s">
         <v>0</v>
@@ -7330,10 +7327,10 @@
         <v>191</v>
       </c>
       <c r="B192" s="11" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="C192" s="14" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="D192" s="18" t="s">
         <v>1</v>
@@ -7347,7 +7344,7 @@
         <v>110</v>
       </c>
       <c r="C193" s="14" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D193" s="18" t="s">
         <v>0</v>
@@ -7361,7 +7358,7 @@
         <v>111</v>
       </c>
       <c r="C194" s="14" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="D194" s="15" t="s">
         <v>1</v>
@@ -7372,10 +7369,10 @@
         <v>194</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="C195" s="14" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="D195" s="19" t="s">
         <v>1</v>
@@ -7386,10 +7383,10 @@
         <v>195</v>
       </c>
       <c r="B196" s="11" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C196" s="14" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="D196" s="20" t="s">
         <v>17</v>
@@ -7403,7 +7400,7 @@
         <v>112</v>
       </c>
       <c r="C197" s="14" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="D197" s="19" t="s">
         <v>1</v>
@@ -7417,7 +7414,7 @@
         <v>113</v>
       </c>
       <c r="C198" s="14" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="D198" s="18" t="s">
         <v>0</v>
@@ -7428,10 +7425,10 @@
         <v>198</v>
       </c>
       <c r="B199" s="11" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="C199" s="14" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="D199" s="18" t="s">
         <v>0</v>
@@ -7442,10 +7439,10 @@
         <v>199</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="C200" s="14" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="D200" s="19" t="s">
         <v>1</v>
@@ -7456,10 +7453,10 @@
         <v>200</v>
       </c>
       <c r="B201" s="11" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="C201" s="14" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="D201" s="24" t="s">
         <v>1</v>
@@ -7473,7 +7470,7 @@
         <v>114</v>
       </c>
       <c r="C202" s="14" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="D202" s="23" t="s">
         <v>20</v>
@@ -7487,7 +7484,7 @@
         <v>115</v>
       </c>
       <c r="C203" s="14" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="D203" s="24" t="s">
         <v>17</v>
@@ -7501,7 +7498,7 @@
         <v>116</v>
       </c>
       <c r="C204" s="14" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D204" s="24" t="s">
         <v>20</v>
@@ -7512,10 +7509,10 @@
         <v>204</v>
       </c>
       <c r="B205" s="11" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="C205" s="14" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D205" s="18" t="s">
         <v>0</v>
@@ -7526,10 +7523,10 @@
         <v>205</v>
       </c>
       <c r="B206" s="11" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="C206" s="14" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="D206" s="18" t="s">
         <v>1</v>
@@ -7543,7 +7540,7 @@
         <v>117</v>
       </c>
       <c r="C207" s="14" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D207" s="19" t="s">
         <v>20</v>
@@ -7554,10 +7551,10 @@
         <v>207</v>
       </c>
       <c r="B208" s="11" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C208" s="14" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="D208" s="18" t="s">
         <v>1</v>
@@ -7568,10 +7565,10 @@
         <v>208</v>
       </c>
       <c r="B209" s="11" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="C209" s="14" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D209" s="18" t="s">
         <v>1</v>
@@ -7582,10 +7579,10 @@
         <v>209</v>
       </c>
       <c r="B210" s="11" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C210" s="14" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D210" s="18" t="s">
         <v>0</v>
@@ -7596,10 +7593,10 @@
         <v>210</v>
       </c>
       <c r="B211" s="11" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="C211" s="14" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="D211" s="32" t="s">
         <v>17</v>
@@ -7610,10 +7607,10 @@
         <v>211</v>
       </c>
       <c r="B212" s="11" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="C212" s="14" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="D212" s="21" t="s">
         <v>0</v>
@@ -7624,10 +7621,10 @@
         <v>212</v>
       </c>
       <c r="B213" s="11" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="C213" s="14" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="D213" s="32" t="s">
         <v>20</v>
@@ -7641,7 +7638,7 @@
         <v>118</v>
       </c>
       <c r="C214" s="14" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="D214" s="21" t="s">
         <v>0</v>
@@ -7655,7 +7652,7 @@
         <v>119</v>
       </c>
       <c r="C215" s="14" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="D215" s="15" t="s">
         <v>20</v>
@@ -7666,10 +7663,10 @@
         <v>215</v>
       </c>
       <c r="B216" s="11" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="C216" s="14" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="D216" s="19" t="s">
         <v>20</v>
@@ -7683,7 +7680,7 @@
         <v>120</v>
       </c>
       <c r="C217" s="14" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="D217" s="18" t="s">
         <v>0</v>
@@ -7697,7 +7694,7 @@
         <v>121</v>
       </c>
       <c r="C218" s="14" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="D218" s="20" t="s">
         <v>20</v>
@@ -7708,10 +7705,10 @@
         <v>218</v>
       </c>
       <c r="B219" s="11" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="C219" s="14" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="D219" s="20" t="s">
         <v>17</v>
@@ -7722,10 +7719,10 @@
         <v>219</v>
       </c>
       <c r="B220" s="11" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="C220" s="14" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="D220" s="19" t="s">
         <v>20</v>
@@ -7739,7 +7736,7 @@
         <v>122</v>
       </c>
       <c r="C221" s="14" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D221" s="18" t="s">
         <v>17</v>
@@ -7753,7 +7750,7 @@
         <v>123</v>
       </c>
       <c r="C222" s="14" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="D222" s="18" t="s">
         <v>0</v>
@@ -7767,7 +7764,7 @@
         <v>124</v>
       </c>
       <c r="C223" s="14" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D223" s="18" t="s">
         <v>0</v>
@@ -7781,7 +7778,7 @@
         <v>125</v>
       </c>
       <c r="C224" s="14" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D224" s="18" t="s">
         <v>0</v>
@@ -7795,7 +7792,7 @@
         <v>126</v>
       </c>
       <c r="C225" s="14" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="D225" s="18" t="s">
         <v>0</v>
@@ -7806,10 +7803,10 @@
         <v>225</v>
       </c>
       <c r="B226" s="11" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="C226" s="14" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="D226" s="18" t="s">
         <v>1</v>
@@ -7823,7 +7820,7 @@
         <v>127</v>
       </c>
       <c r="C227" s="14" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="D227" s="20" t="s">
         <v>17</v>
@@ -7837,7 +7834,7 @@
         <v>128</v>
       </c>
       <c r="C228" s="14" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="D228" s="18" t="s">
         <v>0</v>
@@ -7848,10 +7845,10 @@
         <v>228</v>
       </c>
       <c r="B229" s="11" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C229" s="14" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="D229" s="20" t="s">
         <v>20</v>
@@ -7865,7 +7862,7 @@
         <v>129</v>
       </c>
       <c r="C230" s="14" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="D230" s="20" t="s">
         <v>20</v>
@@ -7879,7 +7876,7 @@
         <v>130</v>
       </c>
       <c r="C231" s="14" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="D231" s="19" t="s">
         <v>1</v>
@@ -7893,7 +7890,7 @@
         <v>131</v>
       </c>
       <c r="C232" s="14" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="D232" s="19" t="s">
         <v>0</v>
@@ -7907,7 +7904,7 @@
         <v>132</v>
       </c>
       <c r="C233" s="14" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="D233" s="20" t="s">
         <v>20</v>
@@ -7921,7 +7918,7 @@
         <v>133</v>
       </c>
       <c r="C234" s="14" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="D234" s="18" t="s">
         <v>0</v>
@@ -7932,10 +7929,10 @@
         <v>234</v>
       </c>
       <c r="B235" s="11" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C235" s="14" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="D235" s="20" t="s">
         <v>17</v>
@@ -7949,7 +7946,7 @@
         <v>134</v>
       </c>
       <c r="C236" s="11" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="D236" s="20" t="s">
         <v>0</v>
@@ -7960,10 +7957,10 @@
         <v>236</v>
       </c>
       <c r="B237" s="16" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C237" s="14" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="D237" s="20" t="s">
         <v>0</v>
@@ -7974,10 +7971,10 @@
         <v>237</v>
       </c>
       <c r="B238" s="11" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="C238" s="14" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="D238" s="18" t="s">
         <v>20</v>
@@ -7991,7 +7988,7 @@
         <v>135</v>
       </c>
       <c r="C239" s="14" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="D239" s="20" t="s">
         <v>0</v>
@@ -8002,10 +7999,10 @@
         <v>239</v>
       </c>
       <c r="B240" s="11" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="C240" s="14" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="D240" s="20" t="s">
         <v>0</v>
@@ -8019,7 +8016,7 @@
         <v>136</v>
       </c>
       <c r="C241" s="14" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="D241" s="21" t="s">
         <v>1</v>
@@ -8030,10 +8027,10 @@
         <v>241</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="C242" s="14" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="D242" s="33" t="s">
         <v>0</v>
@@ -8044,10 +8041,10 @@
         <v>242</v>
       </c>
       <c r="B243" s="11" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C243" s="25" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D243" s="20" t="s">
         <v>20</v>
@@ -8061,7 +8058,7 @@
         <v>137</v>
       </c>
       <c r="C244" s="14" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="D244" s="18" t="s">
         <v>1</v>
@@ -8072,10 +8069,10 @@
         <v>244</v>
       </c>
       <c r="B245" s="11" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="C245" s="14" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="D245" s="18" t="s">
         <v>17</v>
@@ -8086,10 +8083,10 @@
         <v>245</v>
       </c>
       <c r="B246" s="11" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="C246" s="14" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="D246" s="18" t="s">
         <v>17</v>
@@ -8100,10 +8097,10 @@
         <v>246</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C247" s="14" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="D247" s="18" t="s">
         <v>1</v>
@@ -8117,7 +8114,7 @@
         <v>138</v>
       </c>
       <c r="C248" s="14" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="D248" s="18" t="s">
         <v>20</v>
@@ -8128,10 +8125,10 @@
         <v>248</v>
       </c>
       <c r="B249" s="11" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="C249" s="14" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="D249" s="18" t="s">
         <v>20</v>
@@ -8145,7 +8142,7 @@
         <v>139</v>
       </c>
       <c r="C250" s="14" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="D250" s="18" t="s">
         <v>0</v>
@@ -8156,10 +8153,10 @@
         <v>250</v>
       </c>
       <c r="B251" s="11" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="C251" s="14" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="D251" s="19" t="s">
         <v>20</v>
@@ -8173,7 +8170,7 @@
         <v>140</v>
       </c>
       <c r="C252" s="14" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="D252" s="20" t="s">
         <v>20</v>
@@ -8187,7 +8184,7 @@
         <v>141</v>
       </c>
       <c r="C253" s="14" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="D253" s="20" t="s">
         <v>20</v>
@@ -8201,7 +8198,7 @@
         <v>142</v>
       </c>
       <c r="C254" s="14" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="D254" s="20" t="s">
         <v>1</v>
@@ -8212,10 +8209,10 @@
         <v>254</v>
       </c>
       <c r="B255" s="11" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="D255" s="18" t="s">
         <v>20</v>
@@ -8226,10 +8223,10 @@
         <v>255</v>
       </c>
       <c r="B256" s="11" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="C256" s="14" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="D256" s="18" t="s">
         <v>17</v>
@@ -8243,7 +8240,7 @@
         <v>143</v>
       </c>
       <c r="C257" s="14" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="D257" s="19" t="s">
         <v>0</v>
@@ -8257,7 +8254,7 @@
         <v>144</v>
       </c>
       <c r="C258" s="14" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="D258" s="18" t="s">
         <v>0</v>
@@ -8268,10 +8265,10 @@
         <v>258</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="C259" s="14" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D259" s="19" t="s">
         <v>20</v>
@@ -8285,7 +8282,7 @@
         <v>145</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="D260" s="20" t="s">
         <v>1</v>
@@ -8299,7 +8296,7 @@
         <v>146</v>
       </c>
       <c r="C261" s="14" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="D261" s="18" t="s">
         <v>0</v>
@@ -8313,7 +8310,7 @@
         <v>147</v>
       </c>
       <c r="C262" s="14" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="D262" s="19" t="s">
         <v>0</v>
@@ -8327,7 +8324,7 @@
         <v>148</v>
       </c>
       <c r="C263" s="25" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="D263" s="21" t="s">
         <v>0</v>
@@ -8338,10 +8335,10 @@
         <v>263</v>
       </c>
       <c r="B264" s="30" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="C264" s="25" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="D264" s="19" t="s">
         <v>1</v>
@@ -8355,7 +8352,7 @@
         <v>149</v>
       </c>
       <c r="C265" s="25" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="D265" s="18" t="s">
         <v>1</v>
@@ -8369,7 +8366,7 @@
         <v>150</v>
       </c>
       <c r="C266" s="14" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="D266" s="35" t="s">
         <v>1</v>
@@ -8380,10 +8377,10 @@
         <v>266</v>
       </c>
       <c r="B267" s="11" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C267" s="14" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D267" s="18" t="s">
         <v>0</v>
@@ -8394,10 +8391,10 @@
         <v>267</v>
       </c>
       <c r="B268" s="11" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="C268" s="14" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="D268" s="18" t="s">
         <v>1</v>
@@ -8408,10 +8405,10 @@
         <v>268</v>
       </c>
       <c r="B269" s="11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C269" s="14" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="D269" s="18" t="s">
         <v>1</v>
@@ -8425,7 +8422,7 @@
         <v>151</v>
       </c>
       <c r="C270" s="14" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="D270" s="18" t="s">
         <v>1</v>
@@ -8439,7 +8436,7 @@
         <v>152</v>
       </c>
       <c r="C271" s="14" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="D271" s="18" t="s">
         <v>0</v>
@@ -8450,10 +8447,10 @@
         <v>271</v>
       </c>
       <c r="B272" s="11" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="C272" s="14" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="D272" s="18" t="s">
         <v>0</v>
@@ -8467,7 +8464,7 @@
         <v>153</v>
       </c>
       <c r="C273" s="14" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D273" s="15" t="s">
         <v>0</v>
@@ -8481,7 +8478,7 @@
         <v>154</v>
       </c>
       <c r="C274" s="14" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="D274" s="19" t="s">
         <v>20</v>
@@ -8495,7 +8492,7 @@
         <v>155</v>
       </c>
       <c r="C275" s="14" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="D275" s="18" t="s">
         <v>1</v>
@@ -8506,10 +8503,10 @@
         <v>275</v>
       </c>
       <c r="B276" s="11" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C276" s="14" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="D276" s="36" t="s">
         <v>0</v>
@@ -8520,10 +8517,10 @@
         <v>276</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="C277" s="14" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="D277" s="36" t="s">
         <v>20</v>
@@ -8534,10 +8531,10 @@
         <v>277</v>
       </c>
       <c r="B278" s="11" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="C278" s="14" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="D278" s="36" t="s">
         <v>0</v>
@@ -8548,10 +8545,10 @@
         <v>278</v>
       </c>
       <c r="B279" s="11" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="C279" s="14" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="D279" s="36" t="s">
         <v>17</v>
@@ -8562,10 +8559,10 @@
         <v>279</v>
       </c>
       <c r="B280" s="11" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="C280" s="14" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="D280" s="19" t="s">
         <v>20</v>
@@ -8579,7 +8576,7 @@
         <v>156</v>
       </c>
       <c r="C281" s="14" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="D281" s="19" t="s">
         <v>20</v>
@@ -8593,7 +8590,7 @@
         <v>157</v>
       </c>
       <c r="C282" s="14" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="D282" s="19" t="s">
         <v>17</v>
@@ -8607,7 +8604,7 @@
         <v>158</v>
       </c>
       <c r="C283" s="14" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="D283" s="19" t="s">
         <v>20</v>
@@ -8621,7 +8618,7 @@
         <v>159</v>
       </c>
       <c r="C284" s="14" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="D284" s="19" t="s">
         <v>0</v>
@@ -8635,7 +8632,7 @@
         <v>160</v>
       </c>
       <c r="C285" s="14" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="D285" s="19" t="s">
         <v>17</v>
@@ -8649,7 +8646,7 @@
         <v>161</v>
       </c>
       <c r="C286" s="14" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="D286" s="19" t="s">
         <v>17</v>
@@ -8663,7 +8660,7 @@
         <v>162</v>
       </c>
       <c r="C287" s="14" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="D287" s="19" t="s">
         <v>0</v>
@@ -8677,7 +8674,7 @@
         <v>163</v>
       </c>
       <c r="C288" s="14" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="D288" s="19" t="s">
         <v>17</v>
@@ -8691,7 +8688,7 @@
         <v>164</v>
       </c>
       <c r="C289" s="25" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="D289" s="19" t="s">
         <v>17</v>
@@ -8705,7 +8702,7 @@
         <v>165</v>
       </c>
       <c r="C290" s="14" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="D290" s="19" t="s">
         <v>17</v>
@@ -8719,7 +8716,7 @@
         <v>166</v>
       </c>
       <c r="C291" s="14" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="D291" s="19" t="s">
         <v>17</v>
@@ -8730,10 +8727,10 @@
         <v>291</v>
       </c>
       <c r="B292" s="11" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C292" s="14" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="D292" s="8" t="s">
         <v>17</v>
@@ -8744,10 +8741,10 @@
         <v>292</v>
       </c>
       <c r="B293" s="11" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C293" s="14" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="D293" s="19" t="s">
         <v>17</v>
@@ -8758,10 +8755,10 @@
         <v>293</v>
       </c>
       <c r="B294" s="11" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="C294" s="14" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="D294" s="19" t="s">
         <v>20</v>
@@ -8775,7 +8772,7 @@
         <v>167</v>
       </c>
       <c r="C295" s="14" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="D295" s="19" t="s">
         <v>20</v>
@@ -8789,7 +8786,7 @@
         <v>168</v>
       </c>
       <c r="C296" s="14" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="D296" s="19" t="s">
         <v>20</v>
@@ -8803,7 +8800,7 @@
         <v>145</v>
       </c>
       <c r="C297" s="14" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D297" s="19" t="s">
         <v>0</v>
@@ -8817,7 +8814,7 @@
         <v>169</v>
       </c>
       <c r="C298" s="14" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="D298" s="19" t="s">
         <v>1</v>
@@ -8831,7 +8828,7 @@
         <v>170</v>
       </c>
       <c r="C299" s="14" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="D299" s="19" t="s">
         <v>0</v>
@@ -8842,10 +8839,10 @@
         <v>299</v>
       </c>
       <c r="B300" s="11" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C300" s="14" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="D300" s="19" t="s">
         <v>1</v>
@@ -8859,7 +8856,7 @@
         <v>171</v>
       </c>
       <c r="C301" s="14" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="D301" s="15" t="s">
         <v>20</v>
@@ -8870,10 +8867,10 @@
         <v>301</v>
       </c>
       <c r="B302" s="5" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="D302" s="19" t="s">
         <v>0</v>
@@ -8887,7 +8884,7 @@
         <v>172</v>
       </c>
       <c r="C303" s="14" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="D303" s="15" t="s">
         <v>17</v>
@@ -8901,7 +8898,7 @@
         <v>173</v>
       </c>
       <c r="C304" s="14" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="D304" s="19" t="s">
         <v>17</v>
@@ -8915,7 +8912,7 @@
         <v>174</v>
       </c>
       <c r="C305" s="14" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="D305" s="19" t="s">
         <v>17</v>
@@ -8929,7 +8926,7 @@
         <v>175</v>
       </c>
       <c r="C306" s="14" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="D306" s="19" t="s">
         <v>17</v>
@@ -8943,7 +8940,7 @@
         <v>176</v>
       </c>
       <c r="C307" s="14" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="D307" s="15" t="s">
         <v>17</v>
@@ -8957,7 +8954,7 @@
         <v>177</v>
       </c>
       <c r="C308" s="14" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="D308" s="19" t="s">
         <v>17</v>
@@ -8971,7 +8968,7 @@
         <v>178</v>
       </c>
       <c r="C309" s="14" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="D309" s="19" t="s">
         <v>17</v>
@@ -8982,10 +8979,10 @@
         <v>309</v>
       </c>
       <c r="B310" s="11" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="C310" s="14" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="D310" s="19" t="s">
         <v>17</v>
@@ -8996,10 +8993,10 @@
         <v>310</v>
       </c>
       <c r="B311" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="C311" s="14" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="D311" s="19" t="s">
         <v>17</v>
@@ -9013,7 +9010,7 @@
         <v>179</v>
       </c>
       <c r="C312" s="14" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="D312" s="19" t="s">
         <v>17</v>
@@ -9027,7 +9024,7 @@
         <v>180</v>
       </c>
       <c r="C313" s="14" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="D313" s="19" t="s">
         <v>17</v>
@@ -9038,10 +9035,10 @@
         <v>313</v>
       </c>
       <c r="B314" s="11" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="D314" s="19" t="s">
         <v>17</v>
@@ -9055,7 +9052,7 @@
         <v>181</v>
       </c>
       <c r="C315" s="14" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="D315" s="19" t="s">
         <v>0</v>
@@ -9069,7 +9066,7 @@
         <v>182</v>
       </c>
       <c r="C316" s="14" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="D316" s="19" t="s">
         <v>1</v>
@@ -9083,7 +9080,7 @@
         <v>183</v>
       </c>
       <c r="C317" s="14" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="D317" s="18" t="s">
         <v>1</v>
@@ -9094,10 +9091,10 @@
         <v>317</v>
       </c>
       <c r="B318" s="11" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="C318" s="14" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="D318" s="20" t="s">
         <v>17</v>
@@ -9111,7 +9108,7 @@
         <v>184</v>
       </c>
       <c r="C319" s="14" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="D319" s="19" t="s">
         <v>1</v>
@@ -9125,7 +9122,7 @@
         <v>185</v>
       </c>
       <c r="C320" s="14" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="D320" s="19" t="s">
         <v>20</v>
@@ -9139,7 +9136,7 @@
         <v>186</v>
       </c>
       <c r="C321" s="14" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="D321" s="18" t="s">
         <v>20</v>
@@ -9153,7 +9150,7 @@
         <v>187</v>
       </c>
       <c r="C322" s="14" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="D322" s="23" t="s">
         <v>0</v>
@@ -9167,7 +9164,7 @@
         <v>188</v>
       </c>
       <c r="C323" s="14" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="D323" s="22" t="s">
         <v>20</v>
@@ -9181,7 +9178,7 @@
         <v>189</v>
       </c>
       <c r="C324" s="14" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="D324" s="22" t="s">
         <v>20</v>
@@ -9195,7 +9192,7 @@
         <v>190</v>
       </c>
       <c r="C325" s="14" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="D325" s="15" t="s">
         <v>1</v>
@@ -9209,7 +9206,7 @@
         <v>191</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="D326" s="19" t="s">
         <v>20</v>
@@ -9223,7 +9220,7 @@
         <v>192</v>
       </c>
       <c r="C327" s="14" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="D327" s="19" t="s">
         <v>20</v>
@@ -9237,7 +9234,7 @@
         <v>193</v>
       </c>
       <c r="C328" s="14" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="D328" s="19" t="s">
         <v>17</v>
@@ -9248,10 +9245,10 @@
         <v>328</v>
       </c>
       <c r="B329" s="11" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="C329" s="14" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="D329" s="19" t="s">
         <v>17</v>
@@ -9262,10 +9259,10 @@
         <v>329</v>
       </c>
       <c r="B330" s="11" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="C330" s="14" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="D330" s="19" t="s">
         <v>17</v>
@@ -9279,7 +9276,7 @@
         <v>194</v>
       </c>
       <c r="C331" s="14" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="D331" s="19" t="s">
         <v>0</v>
@@ -9290,10 +9287,10 @@
         <v>331</v>
       </c>
       <c r="B332" s="11" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="C332" s="14" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="D332" s="23" t="s">
         <v>0</v>
@@ -9307,7 +9304,7 @@
         <v>5</v>
       </c>
       <c r="C333" s="14" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="D333" s="19" t="s">
         <v>20</v>
@@ -9321,7 +9318,7 @@
         <v>195</v>
       </c>
       <c r="C334" s="14" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="D334" s="19" t="s">
         <v>20</v>
@@ -9332,10 +9329,10 @@
         <v>334</v>
       </c>
       <c r="B335" s="11" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="C335" s="14" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="D335" s="19" t="s">
         <v>20</v>
@@ -9346,10 +9343,10 @@
         <v>335</v>
       </c>
       <c r="B336" s="11" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C336" s="14" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="D336" s="19" t="s">
         <v>20</v>
@@ -9363,7 +9360,7 @@
         <v>196</v>
       </c>
       <c r="C337" s="14" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="D337" s="15" t="s">
         <v>20</v>
@@ -9377,7 +9374,7 @@
         <v>197</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="D338" s="19" t="s">
         <v>1</v>
@@ -9391,7 +9388,7 @@
         <v>198</v>
       </c>
       <c r="C339" s="14" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="D339" s="19" t="s">
         <v>17</v>
@@ -9402,10 +9399,10 @@
         <v>339</v>
       </c>
       <c r="B340" s="11" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="C340" s="14" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="D340" s="19" t="s">
         <v>1</v>
@@ -9419,7 +9416,7 @@
         <v>199</v>
       </c>
       <c r="C341" s="14" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="D341" s="19" t="s">
         <v>1</v>
@@ -9433,7 +9430,7 @@
         <v>200</v>
       </c>
       <c r="C342" s="11" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="D342" s="19" t="s">
         <v>0</v>
@@ -9447,7 +9444,7 @@
         <v>201</v>
       </c>
       <c r="C343" s="11" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="D343" s="19" t="s">
         <v>1</v>
@@ -9461,7 +9458,7 @@
         <v>202</v>
       </c>
       <c r="C344" s="11" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D344" s="19" t="s">
         <v>0</v>
@@ -9475,7 +9472,7 @@
         <v>203</v>
       </c>
       <c r="C345" s="11" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="D345" s="19" t="s">
         <v>17</v>
@@ -9486,10 +9483,10 @@
         <v>345</v>
       </c>
       <c r="B346" s="11" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C346" s="11" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="D346" s="19" t="s">
         <v>17</v>
@@ -9503,7 +9500,7 @@
         <v>204</v>
       </c>
       <c r="C347" s="11" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="D347" s="19" t="s">
         <v>0</v>
@@ -9517,7 +9514,7 @@
         <v>205</v>
       </c>
       <c r="C348" s="11" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="D348" s="19" t="s">
         <v>0</v>
@@ -9531,7 +9528,7 @@
         <v>206</v>
       </c>
       <c r="C349" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="D349" s="19" t="s">
         <v>0</v>
@@ -9545,7 +9542,7 @@
         <v>207</v>
       </c>
       <c r="C350" s="11" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="D350" s="15" t="s">
         <v>1</v>
@@ -9556,10 +9553,10 @@
         <v>350</v>
       </c>
       <c r="B351" s="11" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C351" s="11" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="D351" s="19" t="s">
         <v>1</v>
@@ -9573,7 +9570,7 @@
         <v>208</v>
       </c>
       <c r="C352" s="11" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="D352" s="19" t="s">
         <v>20</v>
@@ -9587,7 +9584,7 @@
         <v>209</v>
       </c>
       <c r="C353" s="11" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="D353" s="19" t="s">
         <v>0</v>
@@ -9598,10 +9595,10 @@
         <v>353</v>
       </c>
       <c r="B354" s="11" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="C354" s="11" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="D354" s="19" t="s">
         <v>20</v>
@@ -9615,7 +9612,7 @@
         <v>210</v>
       </c>
       <c r="C355" s="11" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="D355" s="19" t="s">
         <v>0</v>
@@ -9626,10 +9623,10 @@
         <v>355</v>
       </c>
       <c r="B356" s="11" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="C356" s="11" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="D356" s="19" t="s">
         <v>1</v>
@@ -9643,7 +9640,7 @@
         <v>211</v>
       </c>
       <c r="C357" s="11" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="D357" s="15" t="s">
         <v>20</v>
@@ -9657,7 +9654,7 @@
         <v>6</v>
       </c>
       <c r="C358" s="11" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="D358" s="34" t="s">
         <v>17</v>
@@ -9671,7 +9668,7 @@
         <v>7</v>
       </c>
       <c r="C359" s="30" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="D359" s="30" t="s">
         <v>20</v>
@@ -9682,10 +9679,10 @@
         <v>359</v>
       </c>
       <c r="B360" s="11" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="C360" s="11" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="D360" s="19" t="s">
         <v>17</v>
@@ -9696,10 +9693,10 @@
         <v>360</v>
       </c>
       <c r="B361" s="30" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="C361" s="30" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="D361" s="15" t="s">
         <v>20</v>
@@ -9710,10 +9707,10 @@
         <v>361</v>
       </c>
       <c r="B362" s="30" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="C362" s="30" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="D362" s="15" t="s">
         <v>17</v>
@@ -9727,7 +9724,7 @@
         <v>212</v>
       </c>
       <c r="C363" s="30" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="D363" s="15" t="s">
         <v>20</v>
@@ -9741,7 +9738,7 @@
         <v>213</v>
       </c>
       <c r="C364" s="30" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="D364" s="15" t="s">
         <v>0</v>
@@ -9755,7 +9752,7 @@
         <v>214</v>
       </c>
       <c r="C365" s="30" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="D365" s="15" t="s">
         <v>0</v>
@@ -9769,7 +9766,7 @@
         <v>215</v>
       </c>
       <c r="C366" s="30" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="D366" s="15" t="s">
         <v>20</v>
@@ -9783,7 +9780,7 @@
         <v>216</v>
       </c>
       <c r="C367" s="30" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="D367" s="15" t="s">
         <v>20</v>
@@ -9794,10 +9791,10 @@
         <v>367</v>
       </c>
       <c r="B368" s="11" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="C368" s="30" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="D368" s="15" t="s">
         <v>0</v>
@@ -9811,7 +9808,7 @@
         <v>217</v>
       </c>
       <c r="C369" s="30" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="D369" s="15" t="s">
         <v>20</v>
@@ -9822,10 +9819,10 @@
         <v>369</v>
       </c>
       <c r="B370" s="30" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="C370" s="30" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="D370" s="15" t="s">
         <v>17</v>
@@ -9839,7 +9836,7 @@
         <v>8</v>
       </c>
       <c r="C371" s="30" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="D371" s="15" t="s">
         <v>1</v>
@@ -9853,7 +9850,7 @@
         <v>218</v>
       </c>
       <c r="C372" s="30" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="D372" s="15" t="s">
         <v>0</v>
@@ -9867,7 +9864,7 @@
         <v>219</v>
       </c>
       <c r="C373" s="30" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="D373" s="15" t="s">
         <v>1</v>
@@ -9881,7 +9878,7 @@
         <v>220</v>
       </c>
       <c r="C374" s="30" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="D374" s="15" t="s">
         <v>0</v>
@@ -9895,7 +9892,7 @@
         <v>221</v>
       </c>
       <c r="C375" s="30" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="D375" s="15" t="s">
         <v>1</v>
@@ -9906,10 +9903,10 @@
         <v>375</v>
       </c>
       <c r="B376" s="11" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="C376" s="30" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="D376" s="15" t="s">
         <v>0</v>
@@ -9923,7 +9920,7 @@
         <v>222</v>
       </c>
       <c r="C377" s="30" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="D377" s="15" t="s">
         <v>20</v>
@@ -9937,7 +9934,7 @@
         <v>223</v>
       </c>
       <c r="C378" s="30" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="D378" s="15" t="s">
         <v>17</v>
@@ -9951,7 +9948,7 @@
         <v>224</v>
       </c>
       <c r="C379" s="30" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="D379" s="15" t="s">
         <v>20</v>
@@ -9965,7 +9962,7 @@
         <v>9</v>
       </c>
       <c r="C380" s="30" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="D380" s="15" t="s">
         <v>0</v>
@@ -9976,10 +9973,10 @@
         <v>380</v>
       </c>
       <c r="B381" s="30" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="C381" s="30" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="D381" s="15" t="s">
         <v>17</v>
@@ -9993,7 +9990,7 @@
         <v>225</v>
       </c>
       <c r="C382" s="30" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="D382" s="15" t="s">
         <v>1</v>
@@ -10007,7 +10004,7 @@
         <v>226</v>
       </c>
       <c r="C383" s="30" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="D383" s="15" t="s">
         <v>0</v>
@@ -10021,7 +10018,7 @@
         <v>227</v>
       </c>
       <c r="C384" s="30" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="D384" s="15" t="s">
         <v>0</v>
@@ -10035,7 +10032,7 @@
         <v>228</v>
       </c>
       <c r="C385" s="30" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="D385" s="15" t="s">
         <v>1</v>
@@ -10049,7 +10046,7 @@
         <v>229</v>
       </c>
       <c r="C386" s="11" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="D386" s="15" t="s">
         <v>17</v>
@@ -10063,7 +10060,7 @@
         <v>230</v>
       </c>
       <c r="C387" s="11" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="D387" s="15" t="s">
         <v>20</v>
@@ -10077,7 +10074,7 @@
         <v>231</v>
       </c>
       <c r="C388" s="11" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="D388" s="15" t="s">
         <v>17</v>
@@ -10088,10 +10085,10 @@
         <v>388</v>
       </c>
       <c r="B389" s="11" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="C389" s="11" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="D389" s="19" t="s">
         <v>1</v>
@@ -10102,10 +10099,10 @@
         <v>389</v>
       </c>
       <c r="B390" s="11" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="C390" s="11" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="D390" s="19" t="s">
         <v>1</v>
@@ -10119,7 +10116,7 @@
         <v>232</v>
       </c>
       <c r="C391" s="11" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="D391" s="19" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
chore: sync workbook changes
</commit_message>
<xml_diff>
--- a/data/Ngan-Hang-Cau-Hoi.xlsx
+++ b/data/Ngan-Hang-Cau-Hoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f54d0bdb7235122/Documents/My App/trac-nghiem-luat-dau-thau/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6669B6E6-5ED4-4F8F-B91B-022AC5ED8FA7}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{D1DCDABD-225D-4CEF-B71D-B3A374D525E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C69DD5D-4D78-4F88-9C95-3657EB0C4F3D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0822E189-CD53-41B9-B216-EFA7EF505EBC}"/>
   </bookViews>
@@ -2243,36 +2243,8 @@
 đấu thầu?</t>
   </si>
   <si>
-    <t>A. Chủ đầu tư quyết định xử lý tình huống sau khi có ý kiến của người có thẩm quyền
-B. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của Tổ chuyên gia
-C. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của chủ đầu tư
-D. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của chủ đầu tư và Tổ chuyên
-gia</t>
-  </si>
-  <si>
     <t>Trường hợp một hoặc một số thành viên liên danh vi phạm hợp đồng, không còn năng lực để tiếp tục thực hiện hợp đồng, làm ảnh
 hưởng nghiêm trọng đến tiến độ, chất lượng, hiệu quả của gói thầu thì việc đánh giá uy tín của nhà thầu trong việc thực hiện hợp đồng được xử lý như nào?</t>
-  </si>
-  <si>
-    <t>A. Nhà thầu liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị chủ đầu tư đăng tải thông tin nhà thầu liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
-B.  Chỉ một hoặc một số thành viên liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị chủ đầu tư đăng tải thông tin thành viên liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
-C. Chỉ một hoặc một số thành viên liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị bên mời thầu đăng tải thông tin thành viên liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
-D. Nhà thầu liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị bên mời thầu
-đăng tải thông tin nhà thầu liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia</t>
-  </si>
-  <si>
-    <t>A. Bằng giá trị ghi trong hợp đồng trừ đi giá trị của phần công việc đã thực hiện, được nghiệm thu trước đó
-B. Bằng giá trị ghi trong hợp đồng được cập nhật giá tại thời điểm áp dụng hình thức chỉ định thầu trừ đi giá trị của phần công việc đã thực hiện, được nghiệm thu trước đó
-C. Bằng giá trị của phần công việc còn lại được cập nhật giá tại thời điểm áp dụng hình thức chỉ định thầu
-D. Bằng giá trị ghi trong hợp đồng trừ đi giá trị của phần công việc đã thực hiện trước đó theo dự
-toán được duyệt</t>
-  </si>
-  <si>
-    <t>A. Các thành viên liên danh thỏa thuận, điều chỉnh về phạm vi công việc, tiến độ được rút ngắn và không phải thông báo cho chủ đầu tư
-B. Các thành viên liên danh thỏa thuận, điều chỉnh về phạm vi công việc, tiến độ được rút ngắn và thông báo cho chủ đầu tư
-C. Phải được người có thẩm quyền cho phép chủ đầu tư và nhà thầu thỏa thuận, điều chỉnh phạm vi công việc giữa các thành viên liên danh phù hợp với tiến độ hoặc tiến độ được rút ngắn
-D. Chủ đầu tư và nhà thầu được thỏa thuận điều chỉnh phạm vi công việc giữa các thành viên liên
-danh phù hợp với tiến độ hoặc tiến độ được rút ngắn</t>
   </si>
   <si>
     <t>Trường hợp nhà thầu có nhân sự (ký kết hợp đồng lao động với nhà thầu tại thời điểm nhân sự thực hiện hành vi vi phạm) bị cơ quan điều tra kết luận có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng theo quy định pháp luật về hình sự nhằm mục đích cho nhà thầu trúng thầu nhưng nhân sự của nhà thầu chưa bị
@@ -2536,13 +2508,6 @@
 D. Các đáp án trên đều sai</t>
   </si>
   <si>
-    <t>A. Chịu trách nhiệm về tính chính xác của các thông tin kê khai trên webform và file tài liệu đính
-kèm
-B. Chỉ nộp một bộ E-HSDT đối với một E-TBMT
-C. Chỉ được rút, sửa đổi, nộp lại E-HSDT trước thời điểm đóng thầu
-D. Cả 3 đáp án trên đều đúng</t>
-  </si>
-  <si>
     <t>A. Khi Tổ chuyên gia phát hiện E-HSDT bị lỗi kỹ thuật không mở được
 B. Khi Hệ thống mạng đấu thầu quốc gia gặp sự cố phải tự động gia hạn
 C. Khi E-HSMT được sửa đổi
@@ -2601,20 +2566,6 @@
 nội dung do Hệ thống mạng đấu thầu quốc gia đánh giá "không đạt" thì Tổ chuyên gia không thể sửa đổi kết quả đánh giá từ "không đạt" thành "đạt". Phương án nào sau đây là đúng?</t>
   </si>
   <si>
-    <t>A. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, trạng thái bị tạm ngừng, chấm dứt tham gia Hệ thống mạng đấu thầu quốc gia, doanh thu bình quân hằng năm.
-B. Tư cách hợp lệ, bảo đảm dự thầu, thực hiện nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm
-C. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, trạng thái bị tạm ngừng, chấm dứt tham gia Hệ thống mạng đấu thầu quốc gia, thực hiện nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm
-D. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, lịch sử không hoàn thành hợp đồng do lỗi của nhà thầu, thực hiện
-nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm</t>
-  </si>
-  <si>
-    <t>A. Gói thầu mua sắm hàng hóa áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT đều không có bất kỳ ưu đãi nào
-B. Gói thầu dịch vụ phi tư vấn áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá đánh giá” và các nhà thầu, E-HSDT chào ưu đãi như nhau
-C. Gói thầu xây lắp áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT đều không có bất kỳ ưu đãi nào
-D. Gói thầu máy đặt, máy mượn áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng
-phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT chào ưu đãi như nhau</t>
-  </si>
-  <si>
     <t>Chủ đầu tư yêu cầu gia hạn hiệu lực hồ sơ dự thầu, bảo đảm dự thầu trong trường hợp nào
 sau đây?</t>
   </si>
@@ -2635,13 +2586,6 @@
 D. Phương án A và B đều đúng</t>
   </si>
   <si>
-    <t>A. Thời điểm bắt đầu và kết thúc phải trong giờ hành chính.
-B. Thời điểm bắt đầu không bắt buộc trong giờ hành chính nhưng kết thúc phải trong giờ hành
-chính.
-C. Thời điểm bắt đầu và kết thúc không bắt buộc trong giờ hành chính.
-D. Tất cả phương án trên đều sai</t>
-  </si>
-  <si>
     <t>Đối với gói thầu chào giá trực tuyến rút gọn, nhà thầu xác nhận về việc chấp thuận được
 trao hợp đồng trong thời gian tối đa bao lâu kể từ ngày chủ đầu tư mời nhà thầu xác nhận trên
 Hệ thống mạng đấu thầu quốc gia?</t>
@@ -2684,10 +2628,6 @@
 nhiêu %?</t>
   </si>
   <si>
-    <t>A.80% B.85% C.90%
-D.95%</t>
-  </si>
-  <si>
     <t>A. 5% giá gói thầu
 B. 10% giá gói thầu
 C. 1-3% giá gói thầu
@@ -2698,24 +2638,10 @@
 thế nào?</t>
   </si>
   <si>
-    <t>A. Đề  xuất về tài chính của nhà thầu sẽ bị đánh giá là không đạt
-B. Nhà thầu sẽ bị loại và bị khóa tài khoản trên Hệ thống mạng đấu thầu quốc gia trong vòng 06
-tháng
-C. Hồ sơ dự thầu của nhà thầu sẽ tiếp tục được đánh giá về tài chính căn cứ theo hồ sơ dự thầu đã nộp trước thời điểm đóng thầu
-D. Phương án A và B đều đúng</t>
-  </si>
-  <si>
     <t>A. 100 triệu đồng
 B. 300 triệu đồng
 C. 500 triệu đồng
 D. 01 tỷ đồng</t>
-  </si>
-  <si>
-    <t>A. Đơn vị mua sắm tập trung và các nhà thầu trúng thầu (trong trường hợp không ký thỏa thuận
-khung)
-B. Đơn vị có nhu cầu mua sắm với các nhà thầu trúng thầu (trong trường hợp đơn vị mua sắm tập trung ký thỏa thuận khung với nhà thầu trúng thầu)
-C. Phương án A và B đều đúng
-D. Phương án A và B đều sai</t>
   </si>
   <si>
     <t>A. Gói thầu mua sắm hàng hóa, dịch vụ thuộc dự toán mua sắm có giá gói thầu không quá 500 triệu đồng; gói thầu mua sắm hàng hóa, dịch vụ thuộc dự án có giá gói thầu không quá 01 tỷ đồng
@@ -2810,13 +2736,6 @@
 D. Tất cả các gói thầu áp dụng đấu thầu qua mạng và không qua mạng</t>
   </si>
   <si>
-    <t>A. Đính kèm bản scan báo cáo đánh giá E-HSDT (có chữ ký của tất cả thành viên trong tổ chuyên
-gia)
-B. Đính kèm bản scan báo cáo đánh giá E-HSDT (không cần có chữ ký của tất cả thành viên trong tổ chuyên gia)
-C. Đính kèm bản scan báo cáo đánh giá E-HSDT (chỉ cần chữ ký của tổ trưởng tổ chuyên gia)
-D. Tất cả các phương án đều sai</t>
-  </si>
-  <si>
     <t>Gói thầu hàng hóa có giá gói thầu 02 tỷ đồng thực hiện chào giá trực tuyến theo quy trình rút gọn, trường hợp chủ đầu tư đăng tải thông báo mời thầu vào 11h00 ngày Thứ 2 (15/9/2025), thời điểm nào sau đây là thời
 điểm kết thúc chào giá trực tuyến sớm nhất?</t>
   </si>
@@ -2994,13 +2913,6 @@
 B. Không vượt giá gói thầu, không vượt thời gian thực hiện gói thầu ghi trong hợp đồng và phương pháp, công thức, hạng mục và các nội dung cần thiết để điều chỉnh đã quy định trong hợp đồng
 C. Không vượt thời gian thực hiện gói thầu ghi trong hợp đồng nhưng có thể vượt giá gói thầu
 D. Khi thay đổi thời gian thực hiện hợp đồng nhưng không làm vượt thời gian thực hiện dự án hoặc vượt giá gói thầu (bao gồm dự phòng) được duyệt nhưng không làm vượt tổng mức đầu tư</t>
-  </si>
-  <si>
-    <t>A. Hợp đồng theo đơn giá cố định áp dụng cho gói thầu có thời gian thực hiện dài, hợp đồng theo đơn giá điều chỉnh áp dụng cho gói thầu có thời gian thực hiện ngắn
-B. Đơn giá trong hợp đồng đơn giá cố định không thay đổi, còn đơn giá trong hợp đồng đơn giá điều chỉnh có thể thay đổi
-C. Hợp đồng theo đơn giá cố định không có chi phí dự phòng, còn hợp đồng theo đơn giá điều chỉnh có chi phí dự phòng
-D. Hợp đồng theo đơn giá cố định chỉ áp dụng cho gói thầu dịch vụ tư vấn, hợp đồng theo đơn giá điều chỉnh
-áp dụng cho gói thầu xây lắp</t>
   </si>
   <si>
     <t>So sánh hai tình huống sửa đổi hợp đồng:
@@ -3678,13 +3590,6 @@
 D. Tất cả các phương án trên đều đúng</t>
   </si>
   <si>
-    <t>A. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu Nhật Bản và thành viên này đảm nhận từ 50% trở lên giá trị công việc của gói thầu
-B. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu nội khối và thành viên này đảm nhận từ 25% trở lên giá trị công việc của gói thầu
-C. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu Hoa Kỳ và thành viên này đảm nhận từ 50% trở
-lên giá trị công việc của gói thầu
-D. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu nội khối và thành viên này đảm nhận từ 40% trở lên giá trị công việc của gói thầu</t>
-  </si>
-  <si>
     <t>A. Không ghi rõ số lượng gói thầu
 B.  Không được chia nhỏ gói thầu để tránh áp dụng Nghị định này
 C.  Phải ghi toàn bộ phương thức lựa chọn nhà thầu là đấu thầu qua mạng
@@ -3830,6 +3735,90 @@
 B. Tổ chuyên gia căn cứ theo cataloge, đề xuất kỹ thuật kèm theo để làm cơ sở đánh giá
 C. Hồ sơ dự thầu của nhà thầu không được xem xét, đánh giá
 D. Tiếp tục đánh giá hồ sơ dự thầu, trường hơp nhà thầu trúng thầu thì yêu cầu nhà thầu bổ sung, làm rõ các thông tin này</t>
+  </si>
+  <si>
+    <t>A. Nhà thầu liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị chủ đầu tư đăng tải thông tin nhà thầu liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
+B.  Chỉ một hoặc một số thành viên liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị chủ đầu tư đăng tải thông tin thành viên liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
+C. Chỉ một hoặc một số thành viên liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị bên mời thầu đăng tải thông tin thành viên liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia
+D. Nhà thầu liên danh vi phạm hợp đồng bị coi là không hoàn thành hợp đồng và bị bên mời thầu đăng tải thông tin nhà thầu liên danh vi phạm hợp đồng trên Hệ thống mạng đấu thầu quốc gia</t>
+  </si>
+  <si>
+    <t>A. Bằng giá trị ghi trong hợp đồng trừ đi giá trị của phần công việc đã thực hiện, được nghiệm thu trước đó
+B. Bằng giá trị ghi trong hợp đồng được cập nhật giá tại thời điểm áp dụng hình thức chỉ định thầu trừ đi giá trị của phần công việc đã thực hiện, được nghiệm thu trước đó
+C. Bằng giá trị của phần công việc còn lại được cập nhật giá tại thời điểm áp dụng hình thức chỉ định thầu
+D. Bằng giá trị ghi trong hợp đồng trừ đi giá trị của phần công việc đã thực hiện trước đó theo dự toán được duyệt</t>
+  </si>
+  <si>
+    <t>A. Chủ đầu tư quyết định xử lý tình huống sau khi có ý kiến của người có thẩm quyền
+B. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của Tổ chuyên gia
+C. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của chủ đầu tư
+D. Người có thẩm quyền quyết định xử lý tình huống sau khi có ý kiến của chủ đầu tư và Tổ chuyên gia</t>
+  </si>
+  <si>
+    <t>A. Các thành viên liên danh thỏa thuận, điều chỉnh về phạm vi công việc, tiến độ được rút ngắn và không phải thông báo cho chủ đầu tư
+B. Các thành viên liên danh thỏa thuận, điều chỉnh về phạm vi công việc, tiến độ được rút ngắn và thông báo cho chủ đầu tư
+C. Phải được người có thẩm quyền cho phép chủ đầu tư và nhà thầu thỏa thuận, điều chỉnh phạm vi công việc giữa các thành viên liên danh phù hợp với tiến độ hoặc tiến độ được rút ngắn
+D. Chủ đầu tư và nhà thầu được thỏa thuận điều chỉnh phạm vi công việc giữa các thành viên liên danh phù hợp với tiến độ hoặc tiến độ được rút ngắn</t>
+  </si>
+  <si>
+    <t>A. Chịu trách nhiệm về tính chính xác của các thông tin kê khai trên webform và file tài liệu đính kèm
+B. Chỉ nộp một bộ E-HSDT đối với một E-TBMT
+C. Chỉ được rút, sửa đổi, nộp lại E-HSDT trước thời điểm đóng thầu
+D. Cả 3 đáp án trên đều đúng</t>
+  </si>
+  <si>
+    <t>A. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, trạng thái bị tạm ngừng, chấm dứt tham gia Hệ thống mạng đấu thầu quốc gia, doanh thu bình quân hằng năm.
+B. Tư cách hợp lệ, bảo đảm dự thầu, thực hiện nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm
+C. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, trạng thái bị tạm ngừng, chấm dứt tham gia Hệ thống mạng đấu thầu quốc gia, thực hiện nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm
+D. Tư cách hợp lệ, nhà thầu không có nhân sự bị tòa án kết án có hành vi vi phạm quy định về đấu thầu gây hậu quả nghiêm trọng, lịch sử không hoàn thành hợp đồng do lỗi của nhà thầu, thực hiện nghĩa vụ kê khai thuế và nộp thuế, kết quả hoạt động tài chính, doanh thu bình quân hằng năm</t>
+  </si>
+  <si>
+    <t>A. Gói thầu mua sắm hàng hóa áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT đều không có bất kỳ ưu đãi nào
+B. Gói thầu dịch vụ phi tư vấn áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá đánh giá” và các nhà thầu, E-HSDT chào ưu đãi như nhau
+C. Gói thầu xây lắp áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT đều không có bất kỳ ưu đãi nào
+D. Gói thầu máy đặt, máy mượn áp dụng phương thức một giai đoạn một túi hồ sơ, sử dụng phương pháp “giá thấp nhất” và các nhà thầu, E-HSDT chào ưu đãi như nhau</t>
+  </si>
+  <si>
+    <t>A. Thời điểm bắt đầu và kết thúc phải trong giờ hành chính.
+B. Thời điểm bắt đầu không bắt buộc trong giờ hành chính nhưng kết thúc phải trong giờ hành chính.
+C. Thời điểm bắt đầu và kết thúc không bắt buộc trong giờ hành chính.
+D. Tất cả phương án trên đều sai</t>
+  </si>
+  <si>
+    <t>A.80%
+B.85%
+C.90%
+D.95%</t>
+  </si>
+  <si>
+    <t>A. Đề  xuất về tài chính của nhà thầu sẽ bị đánh giá là không đạt
+B. Nhà thầu sẽ bị loại và bị khóa tài khoản trên Hệ thống mạng đấu thầu quốc gia trong vòng 06 tháng
+C. Hồ sơ dự thầu của nhà thầu sẽ tiếp tục được đánh giá về tài chính căn cứ theo hồ sơ dự thầu đã nộp trước thời điểm đóng thầu
+D. Phương án A và B đều đúng</t>
+  </si>
+  <si>
+    <t>A. Đơn vị mua sắm tập trung và các nhà thầu trúng thầu (trong trường hợp không ký thỏa thuận khung)
+B. Đơn vị có nhu cầu mua sắm với các nhà thầu trúng thầu (trong trường hợp đơn vị mua sắm tập trung ký thỏa thuận khung với nhà thầu trúng thầu)
+C. Phương án A và B đều đúng
+D. Phương án A và B đều sai</t>
+  </si>
+  <si>
+    <t>A. Đính kèm bản scan báo cáo đánh giá E-HSDT (có chữ ký của tất cả thành viên trong tổ chuyên gia)
+B. Đính kèm bản scan báo cáo đánh giá E-HSDT (không cần có chữ ký của tất cả thành viên trong tổ chuyên gia)
+C. Đính kèm bản scan báo cáo đánh giá E-HSDT (chỉ cần chữ ký của tổ trưởng tổ chuyên gia)
+D. Tất cả các phương án đều sai</t>
+  </si>
+  <si>
+    <t>A. Hợp đồng theo đơn giá cố định áp dụng cho gói thầu có thời gian thực hiện dài, hợp đồng theo đơn giá điều chỉnh áp dụng cho gói thầu có thời gian thực hiện ngắn
+B. Đơn giá trong hợp đồng đơn giá cố định không thay đổi, còn đơn giá trong hợp đồng đơn giá điều chỉnh có thể thay đổi
+C. Hợp đồng theo đơn giá cố định không có chi phí dự phòng, còn hợp đồng theo đơn giá điều chỉnh có chi phí dự phòng
+D. Hợp đồng theo đơn giá cố định chỉ áp dụng cho gói thầu dịch vụ tư vấn, hợp đồng theo đơn giá điều chỉnh áp dụng cho gói thầu xây lắp</t>
+  </si>
+  <si>
+    <t>A. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu Nhật Bản và thành viên này đảm nhận từ 50% trở lên giá trị công việc của gói thầu
+B. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu nội khối và thành viên này đảm nhận từ 25% trở lên giá trị công việc của gói thầu
+C. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu Hoa Kỳ và thành viên này đảm nhận từ 50% trở lên giá trị công việc của gói thầu
+D. Nhà thầu liên danh trong đó có thành viên liên danh là nhà thầu nội khối và thành viên này đảm nhận từ 40% trở lên giá trị công việc của gói thầu</t>
   </si>
 </sst>
 </file>
@@ -4185,66 +4174,6 @@
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="96011" y="0"/>
-              </a:lnTo>
-              <a:close/>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:solidFill>
-          <a:srgbClr val="FFFF00">
-            <a:alpha val="50000"/>
-          </a:srgbClr>
-        </a:solidFill>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>7482458</xdr:colOff>
-      <xdr:row>374</xdr:row>
-      <xdr:rowOff>490854</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="105410" cy="175260"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Shape 17">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72FA2F2F-3E30-499B-A18A-D2F82EB7C1DE}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11292458" y="2700654"/>
-          <a:ext cx="105410" cy="175260"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="0" b="0"/>
-          <a:pathLst>
-            <a:path w="105410" h="175260">
-              <a:moveTo>
-                <a:pt x="105155" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="175260"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="105155" y="175260"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="105155" y="0"/>
               </a:lnTo>
               <a:close/>
             </a:path>
@@ -5720,7 +5649,7 @@
         <v>341</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>772</v>
+        <v>758</v>
       </c>
       <c r="D77" s="19" t="s">
         <v>1</v>
@@ -5776,7 +5705,7 @@
         <v>58</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>780</v>
+        <v>766</v>
       </c>
       <c r="D81" s="19" t="s">
         <v>1</v>
@@ -6014,7 +5943,7 @@
         <v>372</v>
       </c>
       <c r="C98" s="25" t="s">
-        <v>783</v>
+        <v>769</v>
       </c>
       <c r="D98" s="20" t="s">
         <v>20</v>
@@ -6042,7 +5971,7 @@
         <v>4</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>773</v>
+        <v>759</v>
       </c>
       <c r="D100" s="26" t="s">
         <v>1</v>
@@ -6056,7 +5985,7 @@
         <v>66</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>779</v>
+        <v>765</v>
       </c>
       <c r="D101" s="21" t="s">
         <v>17</v>
@@ -6140,7 +6069,7 @@
         <v>69</v>
       </c>
       <c r="C107" s="14" t="s">
-        <v>774</v>
+        <v>760</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>20</v>
@@ -6224,7 +6153,7 @@
         <v>389</v>
       </c>
       <c r="C113" s="14" t="s">
-        <v>775</v>
+        <v>761</v>
       </c>
       <c r="D113" s="19" t="s">
         <v>1</v>
@@ -6378,7 +6307,7 @@
         <v>405</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>776</v>
+        <v>762</v>
       </c>
       <c r="D124" s="19" t="s">
         <v>0</v>
@@ -6392,7 +6321,7 @@
         <v>78</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>781</v>
+        <v>767</v>
       </c>
       <c r="D125" s="21" t="s">
         <v>1</v>
@@ -6420,7 +6349,7 @@
         <v>79</v>
       </c>
       <c r="C127" s="14" t="s">
-        <v>782</v>
+        <v>768</v>
       </c>
       <c r="D127" s="21" t="s">
         <v>0</v>
@@ -6602,7 +6531,7 @@
         <v>89</v>
       </c>
       <c r="C140" s="14" t="s">
-        <v>768</v>
+        <v>754</v>
       </c>
       <c r="D140" s="18" t="s">
         <v>17</v>
@@ -6672,7 +6601,7 @@
         <v>93</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>769</v>
+        <v>755</v>
       </c>
       <c r="D145" s="19" t="s">
         <v>17</v>
@@ -6686,7 +6615,7 @@
         <v>428</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>770</v>
+        <v>756</v>
       </c>
       <c r="D146" s="19" t="s">
         <v>20</v>
@@ -6938,7 +6867,7 @@
         <v>456</v>
       </c>
       <c r="C164" s="14" t="s">
-        <v>778</v>
+        <v>764</v>
       </c>
       <c r="D164" s="24" t="s">
         <v>1</v>
@@ -7364,7 +7293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A195" s="7">
         <v>194</v>
       </c>
@@ -7372,27 +7301,27 @@
         <v>504</v>
       </c>
       <c r="C195" s="14" t="s">
-        <v>505</v>
+        <v>772</v>
       </c>
       <c r="D195" s="19" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A196" s="7">
         <v>195</v>
       </c>
       <c r="B196" s="11" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C196" s="14" t="s">
-        <v>507</v>
+        <v>770</v>
       </c>
       <c r="D196" s="20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="197" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A197" s="7">
         <v>196</v>
       </c>
@@ -7400,13 +7329,13 @@
         <v>112</v>
       </c>
       <c r="C197" s="14" t="s">
-        <v>508</v>
+        <v>771</v>
       </c>
       <c r="D197" s="19" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A198" s="10">
         <v>197</v>
       </c>
@@ -7414,7 +7343,7 @@
         <v>113</v>
       </c>
       <c r="C198" s="14" t="s">
-        <v>509</v>
+        <v>773</v>
       </c>
       <c r="D198" s="18" t="s">
         <v>0</v>
@@ -7425,10 +7354,10 @@
         <v>198</v>
       </c>
       <c r="B199" s="11" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="C199" s="14" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="D199" s="18" t="s">
         <v>0</v>
@@ -7439,10 +7368,10 @@
         <v>199</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="C200" s="14" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="D200" s="19" t="s">
         <v>1</v>
@@ -7453,10 +7382,10 @@
         <v>200</v>
       </c>
       <c r="B201" s="11" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="C201" s="14" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="D201" s="24" t="s">
         <v>1</v>
@@ -7470,7 +7399,7 @@
         <v>114</v>
       </c>
       <c r="C202" s="14" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="D202" s="23" t="s">
         <v>20</v>
@@ -7484,7 +7413,7 @@
         <v>115</v>
       </c>
       <c r="C203" s="14" t="s">
-        <v>771</v>
+        <v>757</v>
       </c>
       <c r="D203" s="24" t="s">
         <v>17</v>
@@ -7498,7 +7427,7 @@
         <v>116</v>
       </c>
       <c r="C204" s="14" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="D204" s="24" t="s">
         <v>20</v>
@@ -7509,10 +7438,10 @@
         <v>204</v>
       </c>
       <c r="B205" s="11" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="C205" s="14" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="D205" s="18" t="s">
         <v>0</v>
@@ -7523,10 +7452,10 @@
         <v>205</v>
       </c>
       <c r="B206" s="11" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="C206" s="14" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="D206" s="18" t="s">
         <v>1</v>
@@ -7540,7 +7469,7 @@
         <v>117</v>
       </c>
       <c r="C207" s="14" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="D207" s="19" t="s">
         <v>20</v>
@@ -7551,10 +7480,10 @@
         <v>207</v>
       </c>
       <c r="B208" s="11" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="C208" s="14" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="D208" s="18" t="s">
         <v>1</v>
@@ -7565,10 +7494,10 @@
         <v>208</v>
       </c>
       <c r="B209" s="11" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="C209" s="14" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="D209" s="18" t="s">
         <v>1</v>
@@ -7579,10 +7508,10 @@
         <v>209</v>
       </c>
       <c r="B210" s="11" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="C210" s="14" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="D210" s="18" t="s">
         <v>0</v>
@@ -7593,10 +7522,10 @@
         <v>210</v>
       </c>
       <c r="B211" s="11" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="C211" s="14" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="D211" s="32" t="s">
         <v>17</v>
@@ -7607,10 +7536,10 @@
         <v>211</v>
       </c>
       <c r="B212" s="11" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="C212" s="14" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="D212" s="21" t="s">
         <v>0</v>
@@ -7621,10 +7550,10 @@
         <v>212</v>
       </c>
       <c r="B213" s="11" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="C213" s="14" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="D213" s="32" t="s">
         <v>20</v>
@@ -7638,7 +7567,7 @@
         <v>118</v>
       </c>
       <c r="C214" s="14" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="D214" s="21" t="s">
         <v>0</v>
@@ -7652,7 +7581,7 @@
         <v>119</v>
       </c>
       <c r="C215" s="14" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="D215" s="15" t="s">
         <v>20</v>
@@ -7663,10 +7592,10 @@
         <v>215</v>
       </c>
       <c r="B216" s="11" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="C216" s="14" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="D216" s="19" t="s">
         <v>20</v>
@@ -7680,7 +7609,7 @@
         <v>120</v>
       </c>
       <c r="C217" s="14" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="D217" s="18" t="s">
         <v>0</v>
@@ -7694,7 +7623,7 @@
         <v>121</v>
       </c>
       <c r="C218" s="14" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="D218" s="20" t="s">
         <v>20</v>
@@ -7705,10 +7634,10 @@
         <v>218</v>
       </c>
       <c r="B219" s="11" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="C219" s="14" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="D219" s="20" t="s">
         <v>17</v>
@@ -7719,10 +7648,10 @@
         <v>219</v>
       </c>
       <c r="B220" s="11" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="C220" s="14" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="D220" s="19" t="s">
         <v>20</v>
@@ -7736,7 +7665,7 @@
         <v>122</v>
       </c>
       <c r="C221" s="14" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="D221" s="18" t="s">
         <v>17</v>
@@ -7750,7 +7679,7 @@
         <v>123</v>
       </c>
       <c r="C222" s="14" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="D222" s="18" t="s">
         <v>0</v>
@@ -7764,7 +7693,7 @@
         <v>124</v>
       </c>
       <c r="C223" s="14" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D223" s="18" t="s">
         <v>0</v>
@@ -7778,7 +7707,7 @@
         <v>125</v>
       </c>
       <c r="C224" s="14" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="D224" s="18" t="s">
         <v>0</v>
@@ -7792,7 +7721,7 @@
         <v>126</v>
       </c>
       <c r="C225" s="14" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="D225" s="18" t="s">
         <v>0</v>
@@ -7803,10 +7732,10 @@
         <v>225</v>
       </c>
       <c r="B226" s="11" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="C226" s="14" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="D226" s="18" t="s">
         <v>1</v>
@@ -7820,7 +7749,7 @@
         <v>127</v>
       </c>
       <c r="C227" s="14" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="D227" s="20" t="s">
         <v>17</v>
@@ -7834,7 +7763,7 @@
         <v>128</v>
       </c>
       <c r="C228" s="14" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="D228" s="18" t="s">
         <v>0</v>
@@ -7845,10 +7774,10 @@
         <v>228</v>
       </c>
       <c r="B229" s="11" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="C229" s="14" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="D229" s="20" t="s">
         <v>20</v>
@@ -7862,7 +7791,7 @@
         <v>129</v>
       </c>
       <c r="C230" s="14" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="D230" s="20" t="s">
         <v>20</v>
@@ -7876,13 +7805,13 @@
         <v>130</v>
       </c>
       <c r="C231" s="14" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="D231" s="19" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A232" s="4">
         <v>231</v>
       </c>
@@ -7890,7 +7819,7 @@
         <v>131</v>
       </c>
       <c r="C232" s="14" t="s">
-        <v>558</v>
+        <v>774</v>
       </c>
       <c r="D232" s="19" t="s">
         <v>0</v>
@@ -7904,7 +7833,7 @@
         <v>132</v>
       </c>
       <c r="C233" s="14" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="D233" s="20" t="s">
         <v>20</v>
@@ -7918,7 +7847,7 @@
         <v>133</v>
       </c>
       <c r="C234" s="14" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="D234" s="18" t="s">
         <v>0</v>
@@ -7929,10 +7858,10 @@
         <v>234</v>
       </c>
       <c r="B235" s="11" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="C235" s="14" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="D235" s="20" t="s">
         <v>17</v>
@@ -7946,7 +7875,7 @@
         <v>134</v>
       </c>
       <c r="C236" s="11" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="D236" s="20" t="s">
         <v>0</v>
@@ -7957,10 +7886,10 @@
         <v>236</v>
       </c>
       <c r="B237" s="16" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="C237" s="14" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="D237" s="20" t="s">
         <v>0</v>
@@ -7971,10 +7900,10 @@
         <v>237</v>
       </c>
       <c r="B238" s="11" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="C238" s="14" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="D238" s="18" t="s">
         <v>20</v>
@@ -7988,27 +7917,27 @@
         <v>135</v>
       </c>
       <c r="C239" s="14" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="D239" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A240" s="4">
         <v>239</v>
       </c>
       <c r="B240" s="11" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="C240" s="14" t="s">
-        <v>570</v>
+        <v>775</v>
       </c>
       <c r="D240" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A241" s="4">
         <v>240</v>
       </c>
@@ -8016,7 +7945,7 @@
         <v>136</v>
       </c>
       <c r="C241" s="14" t="s">
-        <v>571</v>
+        <v>776</v>
       </c>
       <c r="D241" s="21" t="s">
         <v>1</v>
@@ -8027,10 +7956,10 @@
         <v>241</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
       <c r="C242" s="14" t="s">
-        <v>573</v>
+        <v>566</v>
       </c>
       <c r="D242" s="33" t="s">
         <v>0</v>
@@ -8041,16 +7970,16 @@
         <v>242</v>
       </c>
       <c r="B243" s="11" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="C243" s="25" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="D243" s="20" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="244" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A244" s="10">
         <v>243</v>
       </c>
@@ -8058,7 +7987,7 @@
         <v>137</v>
       </c>
       <c r="C244" s="14" t="s">
-        <v>576</v>
+        <v>777</v>
       </c>
       <c r="D244" s="18" t="s">
         <v>1</v>
@@ -8069,10 +7998,10 @@
         <v>244</v>
       </c>
       <c r="B245" s="11" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
       <c r="C245" s="14" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
       <c r="D245" s="18" t="s">
         <v>17</v>
@@ -8083,10 +8012,10 @@
         <v>245</v>
       </c>
       <c r="B246" s="11" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
       <c r="C246" s="14" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
       <c r="D246" s="18" t="s">
         <v>17</v>
@@ -8097,10 +8026,10 @@
         <v>246</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
       <c r="C247" s="14" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="D247" s="18" t="s">
         <v>1</v>
@@ -8114,21 +8043,21 @@
         <v>138</v>
       </c>
       <c r="C248" s="14" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
       <c r="D248" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="249" spans="1:4" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A249" s="4">
         <v>248</v>
       </c>
       <c r="B249" s="11" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
       <c r="C249" s="14" t="s">
-        <v>585</v>
+        <v>778</v>
       </c>
       <c r="D249" s="18" t="s">
         <v>20</v>
@@ -8142,21 +8071,21 @@
         <v>139</v>
       </c>
       <c r="C250" s="14" t="s">
-        <v>586</v>
+        <v>577</v>
       </c>
       <c r="D250" s="18" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A251" s="4">
         <v>250</v>
       </c>
       <c r="B251" s="11" t="s">
-        <v>587</v>
+        <v>578</v>
       </c>
       <c r="C251" s="14" t="s">
-        <v>588</v>
+        <v>779</v>
       </c>
       <c r="D251" s="19" t="s">
         <v>20</v>
@@ -8170,13 +8099,13 @@
         <v>140</v>
       </c>
       <c r="C252" s="14" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="D252" s="20" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="253" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A253" s="4">
         <v>252</v>
       </c>
@@ -8184,7 +8113,7 @@
         <v>141</v>
       </c>
       <c r="C253" s="14" t="s">
-        <v>590</v>
+        <v>780</v>
       </c>
       <c r="D253" s="20" t="s">
         <v>20</v>
@@ -8198,7 +8127,7 @@
         <v>142</v>
       </c>
       <c r="C254" s="14" t="s">
-        <v>591</v>
+        <v>580</v>
       </c>
       <c r="D254" s="20" t="s">
         <v>1</v>
@@ -8209,10 +8138,10 @@
         <v>254</v>
       </c>
       <c r="B255" s="11" t="s">
-        <v>592</v>
+        <v>581</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>593</v>
+        <v>582</v>
       </c>
       <c r="D255" s="18" t="s">
         <v>20</v>
@@ -8223,10 +8152,10 @@
         <v>255</v>
       </c>
       <c r="B256" s="11" t="s">
-        <v>594</v>
+        <v>583</v>
       </c>
       <c r="C256" s="14" t="s">
-        <v>595</v>
+        <v>584</v>
       </c>
       <c r="D256" s="18" t="s">
         <v>17</v>
@@ -8240,7 +8169,7 @@
         <v>143</v>
       </c>
       <c r="C257" s="14" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
       <c r="D257" s="19" t="s">
         <v>0</v>
@@ -8254,7 +8183,7 @@
         <v>144</v>
       </c>
       <c r="C258" s="14" t="s">
-        <v>597</v>
+        <v>586</v>
       </c>
       <c r="D258" s="18" t="s">
         <v>0</v>
@@ -8265,10 +8194,10 @@
         <v>258</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>598</v>
+        <v>587</v>
       </c>
       <c r="C259" s="14" t="s">
-        <v>599</v>
+        <v>588</v>
       </c>
       <c r="D259" s="19" t="s">
         <v>20</v>
@@ -8282,7 +8211,7 @@
         <v>145</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>600</v>
+        <v>589</v>
       </c>
       <c r="D260" s="20" t="s">
         <v>1</v>
@@ -8296,7 +8225,7 @@
         <v>146</v>
       </c>
       <c r="C261" s="14" t="s">
-        <v>601</v>
+        <v>590</v>
       </c>
       <c r="D261" s="18" t="s">
         <v>0</v>
@@ -8310,7 +8239,7 @@
         <v>147</v>
       </c>
       <c r="C262" s="14" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="D262" s="19" t="s">
         <v>0</v>
@@ -8324,7 +8253,7 @@
         <v>148</v>
       </c>
       <c r="C263" s="25" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
       <c r="D263" s="21" t="s">
         <v>0</v>
@@ -8335,10 +8264,10 @@
         <v>263</v>
       </c>
       <c r="B264" s="30" t="s">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="C264" s="25" t="s">
-        <v>605</v>
+        <v>594</v>
       </c>
       <c r="D264" s="19" t="s">
         <v>1</v>
@@ -8352,13 +8281,13 @@
         <v>149</v>
       </c>
       <c r="C265" s="25" t="s">
-        <v>606</v>
+        <v>595</v>
       </c>
       <c r="D265" s="18" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A266" s="29">
         <v>265</v>
       </c>
@@ -8366,7 +8295,7 @@
         <v>150</v>
       </c>
       <c r="C266" s="14" t="s">
-        <v>607</v>
+        <v>781</v>
       </c>
       <c r="D266" s="35" t="s">
         <v>1</v>
@@ -8377,10 +8306,10 @@
         <v>266</v>
       </c>
       <c r="B267" s="11" t="s">
-        <v>608</v>
+        <v>596</v>
       </c>
       <c r="C267" s="14" t="s">
-        <v>609</v>
+        <v>597</v>
       </c>
       <c r="D267" s="18" t="s">
         <v>0</v>
@@ -8391,10 +8320,10 @@
         <v>267</v>
       </c>
       <c r="B268" s="11" t="s">
-        <v>610</v>
+        <v>598</v>
       </c>
       <c r="C268" s="14" t="s">
-        <v>611</v>
+        <v>599</v>
       </c>
       <c r="D268" s="18" t="s">
         <v>1</v>
@@ -8405,10 +8334,10 @@
         <v>268</v>
       </c>
       <c r="B269" s="11" t="s">
-        <v>612</v>
+        <v>600</v>
       </c>
       <c r="C269" s="14" t="s">
-        <v>613</v>
+        <v>601</v>
       </c>
       <c r="D269" s="18" t="s">
         <v>1</v>
@@ -8422,7 +8351,7 @@
         <v>151</v>
       </c>
       <c r="C270" s="14" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
       <c r="D270" s="18" t="s">
         <v>1</v>
@@ -8436,7 +8365,7 @@
         <v>152</v>
       </c>
       <c r="C271" s="14" t="s">
-        <v>615</v>
+        <v>603</v>
       </c>
       <c r="D271" s="18" t="s">
         <v>0</v>
@@ -8447,10 +8376,10 @@
         <v>271</v>
       </c>
       <c r="B272" s="11" t="s">
-        <v>616</v>
+        <v>604</v>
       </c>
       <c r="C272" s="14" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="D272" s="18" t="s">
         <v>0</v>
@@ -8464,7 +8393,7 @@
         <v>153</v>
       </c>
       <c r="C273" s="14" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D273" s="15" t="s">
         <v>0</v>
@@ -8478,7 +8407,7 @@
         <v>154</v>
       </c>
       <c r="C274" s="14" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="D274" s="19" t="s">
         <v>20</v>
@@ -8492,7 +8421,7 @@
         <v>155</v>
       </c>
       <c r="C275" s="14" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
       <c r="D275" s="18" t="s">
         <v>1</v>
@@ -8503,10 +8432,10 @@
         <v>275</v>
       </c>
       <c r="B276" s="11" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="C276" s="14" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
       <c r="D276" s="36" t="s">
         <v>0</v>
@@ -8517,10 +8446,10 @@
         <v>276</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>623</v>
+        <v>611</v>
       </c>
       <c r="C277" s="14" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
       <c r="D277" s="36" t="s">
         <v>20</v>
@@ -8531,10 +8460,10 @@
         <v>277</v>
       </c>
       <c r="B278" s="11" t="s">
-        <v>625</v>
+        <v>613</v>
       </c>
       <c r="C278" s="14" t="s">
-        <v>626</v>
+        <v>614</v>
       </c>
       <c r="D278" s="36" t="s">
         <v>0</v>
@@ -8545,10 +8474,10 @@
         <v>278</v>
       </c>
       <c r="B279" s="11" t="s">
-        <v>767</v>
+        <v>753</v>
       </c>
       <c r="C279" s="14" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="D279" s="36" t="s">
         <v>17</v>
@@ -8559,10 +8488,10 @@
         <v>279</v>
       </c>
       <c r="B280" s="11" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="C280" s="14" t="s">
-        <v>629</v>
+        <v>617</v>
       </c>
       <c r="D280" s="19" t="s">
         <v>20</v>
@@ -8576,7 +8505,7 @@
         <v>156</v>
       </c>
       <c r="C281" s="14" t="s">
-        <v>630</v>
+        <v>618</v>
       </c>
       <c r="D281" s="19" t="s">
         <v>20</v>
@@ -8590,7 +8519,7 @@
         <v>157</v>
       </c>
       <c r="C282" s="14" t="s">
-        <v>631</v>
+        <v>619</v>
       </c>
       <c r="D282" s="19" t="s">
         <v>17</v>
@@ -8604,7 +8533,7 @@
         <v>158</v>
       </c>
       <c r="C283" s="14" t="s">
-        <v>632</v>
+        <v>620</v>
       </c>
       <c r="D283" s="19" t="s">
         <v>20</v>
@@ -8618,7 +8547,7 @@
         <v>159</v>
       </c>
       <c r="C284" s="14" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
       <c r="D284" s="19" t="s">
         <v>0</v>
@@ -8632,7 +8561,7 @@
         <v>160</v>
       </c>
       <c r="C285" s="14" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
       <c r="D285" s="19" t="s">
         <v>17</v>
@@ -8646,7 +8575,7 @@
         <v>161</v>
       </c>
       <c r="C286" s="14" t="s">
-        <v>635</v>
+        <v>623</v>
       </c>
       <c r="D286" s="19" t="s">
         <v>17</v>
@@ -8660,7 +8589,7 @@
         <v>162</v>
       </c>
       <c r="C287" s="14" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="D287" s="19" t="s">
         <v>0</v>
@@ -8674,7 +8603,7 @@
         <v>163</v>
       </c>
       <c r="C288" s="14" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D288" s="19" t="s">
         <v>17</v>
@@ -8688,7 +8617,7 @@
         <v>164</v>
       </c>
       <c r="C289" s="25" t="s">
-        <v>638</v>
+        <v>626</v>
       </c>
       <c r="D289" s="19" t="s">
         <v>17</v>
@@ -8702,13 +8631,13 @@
         <v>165</v>
       </c>
       <c r="C290" s="14" t="s">
-        <v>639</v>
+        <v>627</v>
       </c>
       <c r="D290" s="19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="291" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A291" s="4">
         <v>290</v>
       </c>
@@ -8716,7 +8645,7 @@
         <v>166</v>
       </c>
       <c r="C291" s="14" t="s">
-        <v>640</v>
+        <v>782</v>
       </c>
       <c r="D291" s="19" t="s">
         <v>17</v>
@@ -8727,10 +8656,10 @@
         <v>291</v>
       </c>
       <c r="B292" s="11" t="s">
-        <v>641</v>
+        <v>628</v>
       </c>
       <c r="C292" s="14" t="s">
-        <v>642</v>
+        <v>629</v>
       </c>
       <c r="D292" s="8" t="s">
         <v>17</v>
@@ -8741,10 +8670,10 @@
         <v>292</v>
       </c>
       <c r="B293" s="11" t="s">
-        <v>643</v>
+        <v>630</v>
       </c>
       <c r="C293" s="14" t="s">
-        <v>644</v>
+        <v>631</v>
       </c>
       <c r="D293" s="19" t="s">
         <v>17</v>
@@ -8755,10 +8684,10 @@
         <v>293</v>
       </c>
       <c r="B294" s="11" t="s">
-        <v>645</v>
+        <v>632</v>
       </c>
       <c r="C294" s="14" t="s">
-        <v>646</v>
+        <v>633</v>
       </c>
       <c r="D294" s="19" t="s">
         <v>20</v>
@@ -8772,7 +8701,7 @@
         <v>167</v>
       </c>
       <c r="C295" s="14" t="s">
-        <v>647</v>
+        <v>634</v>
       </c>
       <c r="D295" s="19" t="s">
         <v>20</v>
@@ -8786,7 +8715,7 @@
         <v>168</v>
       </c>
       <c r="C296" s="14" t="s">
-        <v>648</v>
+        <v>635</v>
       </c>
       <c r="D296" s="19" t="s">
         <v>20</v>
@@ -8800,7 +8729,7 @@
         <v>145</v>
       </c>
       <c r="C297" s="14" t="s">
-        <v>649</v>
+        <v>636</v>
       </c>
       <c r="D297" s="19" t="s">
         <v>0</v>
@@ -8814,7 +8743,7 @@
         <v>169</v>
       </c>
       <c r="C298" s="14" t="s">
-        <v>650</v>
+        <v>637</v>
       </c>
       <c r="D298" s="19" t="s">
         <v>1</v>
@@ -8828,7 +8757,7 @@
         <v>170</v>
       </c>
       <c r="C299" s="14" t="s">
-        <v>651</v>
+        <v>638</v>
       </c>
       <c r="D299" s="19" t="s">
         <v>0</v>
@@ -8839,10 +8768,10 @@
         <v>299</v>
       </c>
       <c r="B300" s="11" t="s">
-        <v>652</v>
+        <v>639</v>
       </c>
       <c r="C300" s="14" t="s">
-        <v>653</v>
+        <v>640</v>
       </c>
       <c r="D300" s="19" t="s">
         <v>1</v>
@@ -8856,7 +8785,7 @@
         <v>171</v>
       </c>
       <c r="C301" s="14" t="s">
-        <v>654</v>
+        <v>641</v>
       </c>
       <c r="D301" s="15" t="s">
         <v>20</v>
@@ -8867,10 +8796,10 @@
         <v>301</v>
       </c>
       <c r="B302" s="5" t="s">
-        <v>655</v>
+        <v>642</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>656</v>
+        <v>643</v>
       </c>
       <c r="D302" s="19" t="s">
         <v>0</v>
@@ -8884,7 +8813,7 @@
         <v>172</v>
       </c>
       <c r="C303" s="14" t="s">
-        <v>657</v>
+        <v>644</v>
       </c>
       <c r="D303" s="15" t="s">
         <v>17</v>
@@ -8898,7 +8827,7 @@
         <v>173</v>
       </c>
       <c r="C304" s="14" t="s">
-        <v>658</v>
+        <v>645</v>
       </c>
       <c r="D304" s="19" t="s">
         <v>17</v>
@@ -8912,7 +8841,7 @@
         <v>174</v>
       </c>
       <c r="C305" s="14" t="s">
-        <v>659</v>
+        <v>646</v>
       </c>
       <c r="D305" s="19" t="s">
         <v>17</v>
@@ -8926,7 +8855,7 @@
         <v>175</v>
       </c>
       <c r="C306" s="14" t="s">
-        <v>660</v>
+        <v>647</v>
       </c>
       <c r="D306" s="19" t="s">
         <v>17</v>
@@ -8940,7 +8869,7 @@
         <v>176</v>
       </c>
       <c r="C307" s="14" t="s">
-        <v>661</v>
+        <v>648</v>
       </c>
       <c r="D307" s="15" t="s">
         <v>17</v>
@@ -8954,7 +8883,7 @@
         <v>177</v>
       </c>
       <c r="C308" s="14" t="s">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="D308" s="19" t="s">
         <v>17</v>
@@ -8968,7 +8897,7 @@
         <v>178</v>
       </c>
       <c r="C309" s="14" t="s">
-        <v>663</v>
+        <v>650</v>
       </c>
       <c r="D309" s="19" t="s">
         <v>17</v>
@@ -8979,10 +8908,10 @@
         <v>309</v>
       </c>
       <c r="B310" s="11" t="s">
-        <v>664</v>
+        <v>651</v>
       </c>
       <c r="C310" s="14" t="s">
-        <v>665</v>
+        <v>652</v>
       </c>
       <c r="D310" s="19" t="s">
         <v>17</v>
@@ -8993,10 +8922,10 @@
         <v>310</v>
       </c>
       <c r="B311" s="11" t="s">
-        <v>666</v>
+        <v>653</v>
       </c>
       <c r="C311" s="14" t="s">
-        <v>663</v>
+        <v>650</v>
       </c>
       <c r="D311" s="19" t="s">
         <v>17</v>
@@ -9010,7 +8939,7 @@
         <v>179</v>
       </c>
       <c r="C312" s="14" t="s">
-        <v>667</v>
+        <v>654</v>
       </c>
       <c r="D312" s="19" t="s">
         <v>17</v>
@@ -9024,7 +8953,7 @@
         <v>180</v>
       </c>
       <c r="C313" s="14" t="s">
-        <v>668</v>
+        <v>655</v>
       </c>
       <c r="D313" s="19" t="s">
         <v>17</v>
@@ -9035,10 +8964,10 @@
         <v>313</v>
       </c>
       <c r="B314" s="11" t="s">
-        <v>669</v>
+        <v>656</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>670</v>
+        <v>657</v>
       </c>
       <c r="D314" s="19" t="s">
         <v>17</v>
@@ -9052,7 +8981,7 @@
         <v>181</v>
       </c>
       <c r="C315" s="14" t="s">
-        <v>671</v>
+        <v>658</v>
       </c>
       <c r="D315" s="19" t="s">
         <v>0</v>
@@ -9066,7 +8995,7 @@
         <v>182</v>
       </c>
       <c r="C316" s="14" t="s">
-        <v>672</v>
+        <v>659</v>
       </c>
       <c r="D316" s="19" t="s">
         <v>1</v>
@@ -9080,7 +9009,7 @@
         <v>183</v>
       </c>
       <c r="C317" s="14" t="s">
-        <v>673</v>
+        <v>660</v>
       </c>
       <c r="D317" s="18" t="s">
         <v>1</v>
@@ -9091,10 +9020,10 @@
         <v>317</v>
       </c>
       <c r="B318" s="11" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="C318" s="14" t="s">
-        <v>675</v>
+        <v>662</v>
       </c>
       <c r="D318" s="20" t="s">
         <v>17</v>
@@ -9108,7 +9037,7 @@
         <v>184</v>
       </c>
       <c r="C319" s="14" t="s">
-        <v>676</v>
+        <v>663</v>
       </c>
       <c r="D319" s="19" t="s">
         <v>1</v>
@@ -9122,7 +9051,7 @@
         <v>185</v>
       </c>
       <c r="C320" s="14" t="s">
-        <v>677</v>
+        <v>664</v>
       </c>
       <c r="D320" s="19" t="s">
         <v>20</v>
@@ -9136,7 +9065,7 @@
         <v>186</v>
       </c>
       <c r="C321" s="14" t="s">
-        <v>678</v>
+        <v>665</v>
       </c>
       <c r="D321" s="18" t="s">
         <v>20</v>
@@ -9150,7 +9079,7 @@
         <v>187</v>
       </c>
       <c r="C322" s="14" t="s">
-        <v>679</v>
+        <v>666</v>
       </c>
       <c r="D322" s="23" t="s">
         <v>0</v>
@@ -9164,7 +9093,7 @@
         <v>188</v>
       </c>
       <c r="C323" s="14" t="s">
-        <v>680</v>
+        <v>667</v>
       </c>
       <c r="D323" s="22" t="s">
         <v>20</v>
@@ -9178,7 +9107,7 @@
         <v>189</v>
       </c>
       <c r="C324" s="14" t="s">
-        <v>681</v>
+        <v>668</v>
       </c>
       <c r="D324" s="22" t="s">
         <v>20</v>
@@ -9192,7 +9121,7 @@
         <v>190</v>
       </c>
       <c r="C325" s="14" t="s">
-        <v>682</v>
+        <v>669</v>
       </c>
       <c r="D325" s="15" t="s">
         <v>1</v>
@@ -9206,7 +9135,7 @@
         <v>191</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>683</v>
+        <v>670</v>
       </c>
       <c r="D326" s="19" t="s">
         <v>20</v>
@@ -9220,7 +9149,7 @@
         <v>192</v>
       </c>
       <c r="C327" s="14" t="s">
-        <v>684</v>
+        <v>671</v>
       </c>
       <c r="D327" s="19" t="s">
         <v>20</v>
@@ -9234,7 +9163,7 @@
         <v>193</v>
       </c>
       <c r="C328" s="14" t="s">
-        <v>685</v>
+        <v>672</v>
       </c>
       <c r="D328" s="19" t="s">
         <v>17</v>
@@ -9245,10 +9174,10 @@
         <v>328</v>
       </c>
       <c r="B329" s="11" t="s">
-        <v>686</v>
+        <v>673</v>
       </c>
       <c r="C329" s="14" t="s">
-        <v>687</v>
+        <v>674</v>
       </c>
       <c r="D329" s="19" t="s">
         <v>17</v>
@@ -9259,10 +9188,10 @@
         <v>329</v>
       </c>
       <c r="B330" s="11" t="s">
-        <v>688</v>
+        <v>675</v>
       </c>
       <c r="C330" s="14" t="s">
-        <v>689</v>
+        <v>676</v>
       </c>
       <c r="D330" s="19" t="s">
         <v>17</v>
@@ -9276,7 +9205,7 @@
         <v>194</v>
       </c>
       <c r="C331" s="14" t="s">
-        <v>690</v>
+        <v>677</v>
       </c>
       <c r="D331" s="19" t="s">
         <v>0</v>
@@ -9287,10 +9216,10 @@
         <v>331</v>
       </c>
       <c r="B332" s="11" t="s">
-        <v>691</v>
+        <v>678</v>
       </c>
       <c r="C332" s="14" t="s">
-        <v>692</v>
+        <v>679</v>
       </c>
       <c r="D332" s="23" t="s">
         <v>0</v>
@@ -9304,7 +9233,7 @@
         <v>5</v>
       </c>
       <c r="C333" s="14" t="s">
-        <v>693</v>
+        <v>680</v>
       </c>
       <c r="D333" s="19" t="s">
         <v>20</v>
@@ -9318,7 +9247,7 @@
         <v>195</v>
       </c>
       <c r="C334" s="14" t="s">
-        <v>694</v>
+        <v>681</v>
       </c>
       <c r="D334" s="19" t="s">
         <v>20</v>
@@ -9329,10 +9258,10 @@
         <v>334</v>
       </c>
       <c r="B335" s="11" t="s">
-        <v>695</v>
+        <v>682</v>
       </c>
       <c r="C335" s="14" t="s">
-        <v>696</v>
+        <v>683</v>
       </c>
       <c r="D335" s="19" t="s">
         <v>20</v>
@@ -9343,10 +9272,10 @@
         <v>335</v>
       </c>
       <c r="B336" s="11" t="s">
-        <v>697</v>
+        <v>684</v>
       </c>
       <c r="C336" s="14" t="s">
-        <v>698</v>
+        <v>685</v>
       </c>
       <c r="D336" s="19" t="s">
         <v>20</v>
@@ -9360,7 +9289,7 @@
         <v>196</v>
       </c>
       <c r="C337" s="14" t="s">
-        <v>699</v>
+        <v>686</v>
       </c>
       <c r="D337" s="15" t="s">
         <v>20</v>
@@ -9374,7 +9303,7 @@
         <v>197</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>700</v>
+        <v>687</v>
       </c>
       <c r="D338" s="19" t="s">
         <v>1</v>
@@ -9388,7 +9317,7 @@
         <v>198</v>
       </c>
       <c r="C339" s="14" t="s">
-        <v>701</v>
+        <v>688</v>
       </c>
       <c r="D339" s="19" t="s">
         <v>17</v>
@@ -9399,10 +9328,10 @@
         <v>339</v>
       </c>
       <c r="B340" s="11" t="s">
-        <v>702</v>
+        <v>689</v>
       </c>
       <c r="C340" s="14" t="s">
-        <v>703</v>
+        <v>690</v>
       </c>
       <c r="D340" s="19" t="s">
         <v>1</v>
@@ -9416,7 +9345,7 @@
         <v>199</v>
       </c>
       <c r="C341" s="14" t="s">
-        <v>704</v>
+        <v>691</v>
       </c>
       <c r="D341" s="19" t="s">
         <v>1</v>
@@ -9430,7 +9359,7 @@
         <v>200</v>
       </c>
       <c r="C342" s="11" t="s">
-        <v>705</v>
+        <v>692</v>
       </c>
       <c r="D342" s="19" t="s">
         <v>0</v>
@@ -9444,7 +9373,7 @@
         <v>201</v>
       </c>
       <c r="C343" s="11" t="s">
-        <v>706</v>
+        <v>693</v>
       </c>
       <c r="D343" s="19" t="s">
         <v>1</v>
@@ -9458,7 +9387,7 @@
         <v>202</v>
       </c>
       <c r="C344" s="11" t="s">
-        <v>777</v>
+        <v>763</v>
       </c>
       <c r="D344" s="19" t="s">
         <v>0</v>
@@ -9472,7 +9401,7 @@
         <v>203</v>
       </c>
       <c r="C345" s="11" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="D345" s="19" t="s">
         <v>17</v>
@@ -9483,10 +9412,10 @@
         <v>345</v>
       </c>
       <c r="B346" s="11" t="s">
-        <v>708</v>
+        <v>695</v>
       </c>
       <c r="C346" s="11" t="s">
-        <v>709</v>
+        <v>696</v>
       </c>
       <c r="D346" s="19" t="s">
         <v>17</v>
@@ -9500,7 +9429,7 @@
         <v>204</v>
       </c>
       <c r="C347" s="11" t="s">
-        <v>710</v>
+        <v>697</v>
       </c>
       <c r="D347" s="19" t="s">
         <v>0</v>
@@ -9514,7 +9443,7 @@
         <v>205</v>
       </c>
       <c r="C348" s="11" t="s">
-        <v>711</v>
+        <v>698</v>
       </c>
       <c r="D348" s="19" t="s">
         <v>0</v>
@@ -9528,7 +9457,7 @@
         <v>206</v>
       </c>
       <c r="C349" s="11" t="s">
-        <v>712</v>
+        <v>699</v>
       </c>
       <c r="D349" s="19" t="s">
         <v>0</v>
@@ -9542,7 +9471,7 @@
         <v>207</v>
       </c>
       <c r="C350" s="11" t="s">
-        <v>713</v>
+        <v>700</v>
       </c>
       <c r="D350" s="15" t="s">
         <v>1</v>
@@ -9553,10 +9482,10 @@
         <v>350</v>
       </c>
       <c r="B351" s="11" t="s">
-        <v>714</v>
+        <v>701</v>
       </c>
       <c r="C351" s="11" t="s">
-        <v>715</v>
+        <v>702</v>
       </c>
       <c r="D351" s="19" t="s">
         <v>1</v>
@@ -9570,7 +9499,7 @@
         <v>208</v>
       </c>
       <c r="C352" s="11" t="s">
-        <v>716</v>
+        <v>703</v>
       </c>
       <c r="D352" s="19" t="s">
         <v>20</v>
@@ -9584,7 +9513,7 @@
         <v>209</v>
       </c>
       <c r="C353" s="11" t="s">
-        <v>717</v>
+        <v>704</v>
       </c>
       <c r="D353" s="19" t="s">
         <v>0</v>
@@ -9595,10 +9524,10 @@
         <v>353</v>
       </c>
       <c r="B354" s="11" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="C354" s="11" t="s">
-        <v>719</v>
+        <v>706</v>
       </c>
       <c r="D354" s="19" t="s">
         <v>20</v>
@@ -9612,7 +9541,7 @@
         <v>210</v>
       </c>
       <c r="C355" s="11" t="s">
-        <v>720</v>
+        <v>707</v>
       </c>
       <c r="D355" s="19" t="s">
         <v>0</v>
@@ -9623,10 +9552,10 @@
         <v>355</v>
       </c>
       <c r="B356" s="11" t="s">
-        <v>721</v>
+        <v>708</v>
       </c>
       <c r="C356" s="11" t="s">
-        <v>722</v>
+        <v>709</v>
       </c>
       <c r="D356" s="19" t="s">
         <v>1</v>
@@ -9640,7 +9569,7 @@
         <v>211</v>
       </c>
       <c r="C357" s="11" t="s">
-        <v>723</v>
+        <v>710</v>
       </c>
       <c r="D357" s="15" t="s">
         <v>20</v>
@@ -9654,7 +9583,7 @@
         <v>6</v>
       </c>
       <c r="C358" s="11" t="s">
-        <v>724</v>
+        <v>711</v>
       </c>
       <c r="D358" s="34" t="s">
         <v>17</v>
@@ -9668,7 +9597,7 @@
         <v>7</v>
       </c>
       <c r="C359" s="30" t="s">
-        <v>725</v>
+        <v>712</v>
       </c>
       <c r="D359" s="30" t="s">
         <v>20</v>
@@ -9679,10 +9608,10 @@
         <v>359</v>
       </c>
       <c r="B360" s="11" t="s">
-        <v>726</v>
+        <v>713</v>
       </c>
       <c r="C360" s="11" t="s">
-        <v>727</v>
+        <v>714</v>
       </c>
       <c r="D360" s="19" t="s">
         <v>17</v>
@@ -9693,10 +9622,10 @@
         <v>360</v>
       </c>
       <c r="B361" s="30" t="s">
-        <v>728</v>
+        <v>715</v>
       </c>
       <c r="C361" s="30" t="s">
-        <v>729</v>
+        <v>716</v>
       </c>
       <c r="D361" s="15" t="s">
         <v>20</v>
@@ -9707,10 +9636,10 @@
         <v>361</v>
       </c>
       <c r="B362" s="30" t="s">
-        <v>730</v>
+        <v>717</v>
       </c>
       <c r="C362" s="30" t="s">
-        <v>731</v>
+        <v>718</v>
       </c>
       <c r="D362" s="15" t="s">
         <v>17</v>
@@ -9724,7 +9653,7 @@
         <v>212</v>
       </c>
       <c r="C363" s="30" t="s">
-        <v>732</v>
+        <v>719</v>
       </c>
       <c r="D363" s="15" t="s">
         <v>20</v>
@@ -9738,7 +9667,7 @@
         <v>213</v>
       </c>
       <c r="C364" s="30" t="s">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="D364" s="15" t="s">
         <v>0</v>
@@ -9752,7 +9681,7 @@
         <v>214</v>
       </c>
       <c r="C365" s="30" t="s">
-        <v>734</v>
+        <v>721</v>
       </c>
       <c r="D365" s="15" t="s">
         <v>0</v>
@@ -9766,7 +9695,7 @@
         <v>215</v>
       </c>
       <c r="C366" s="30" t="s">
-        <v>735</v>
+        <v>722</v>
       </c>
       <c r="D366" s="15" t="s">
         <v>20</v>
@@ -9780,7 +9709,7 @@
         <v>216</v>
       </c>
       <c r="C367" s="30" t="s">
-        <v>736</v>
+        <v>723</v>
       </c>
       <c r="D367" s="15" t="s">
         <v>20</v>
@@ -9791,10 +9720,10 @@
         <v>367</v>
       </c>
       <c r="B368" s="11" t="s">
-        <v>737</v>
+        <v>724</v>
       </c>
       <c r="C368" s="30" t="s">
-        <v>738</v>
+        <v>725</v>
       </c>
       <c r="D368" s="15" t="s">
         <v>0</v>
@@ -9808,7 +9737,7 @@
         <v>217</v>
       </c>
       <c r="C369" s="30" t="s">
-        <v>739</v>
+        <v>726</v>
       </c>
       <c r="D369" s="15" t="s">
         <v>20</v>
@@ -9819,10 +9748,10 @@
         <v>369</v>
       </c>
       <c r="B370" s="30" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="C370" s="30" t="s">
-        <v>741</v>
+        <v>728</v>
       </c>
       <c r="D370" s="15" t="s">
         <v>17</v>
@@ -9836,7 +9765,7 @@
         <v>8</v>
       </c>
       <c r="C371" s="30" t="s">
-        <v>742</v>
+        <v>729</v>
       </c>
       <c r="D371" s="15" t="s">
         <v>1</v>
@@ -9850,7 +9779,7 @@
         <v>218</v>
       </c>
       <c r="C372" s="30" t="s">
-        <v>743</v>
+        <v>730</v>
       </c>
       <c r="D372" s="15" t="s">
         <v>0</v>
@@ -9864,7 +9793,7 @@
         <v>219</v>
       </c>
       <c r="C373" s="30" t="s">
-        <v>744</v>
+        <v>731</v>
       </c>
       <c r="D373" s="15" t="s">
         <v>1</v>
@@ -9878,7 +9807,7 @@
         <v>220</v>
       </c>
       <c r="C374" s="30" t="s">
-        <v>745</v>
+        <v>732</v>
       </c>
       <c r="D374" s="15" t="s">
         <v>0</v>
@@ -9892,7 +9821,7 @@
         <v>221</v>
       </c>
       <c r="C375" s="30" t="s">
-        <v>746</v>
+        <v>733</v>
       </c>
       <c r="D375" s="15" t="s">
         <v>1</v>
@@ -9903,10 +9832,10 @@
         <v>375</v>
       </c>
       <c r="B376" s="11" t="s">
-        <v>747</v>
+        <v>734</v>
       </c>
       <c r="C376" s="30" t="s">
-        <v>748</v>
+        <v>735</v>
       </c>
       <c r="D376" s="15" t="s">
         <v>0</v>
@@ -9920,7 +9849,7 @@
         <v>222</v>
       </c>
       <c r="C377" s="30" t="s">
-        <v>749</v>
+        <v>736</v>
       </c>
       <c r="D377" s="15" t="s">
         <v>20</v>
@@ -9934,7 +9863,7 @@
         <v>223</v>
       </c>
       <c r="C378" s="30" t="s">
-        <v>750</v>
+        <v>737</v>
       </c>
       <c r="D378" s="15" t="s">
         <v>17</v>
@@ -9948,7 +9877,7 @@
         <v>224</v>
       </c>
       <c r="C379" s="30" t="s">
-        <v>751</v>
+        <v>738</v>
       </c>
       <c r="D379" s="15" t="s">
         <v>20</v>
@@ -9962,7 +9891,7 @@
         <v>9</v>
       </c>
       <c r="C380" s="30" t="s">
-        <v>752</v>
+        <v>739</v>
       </c>
       <c r="D380" s="15" t="s">
         <v>0</v>
@@ -9973,10 +9902,10 @@
         <v>380</v>
       </c>
       <c r="B381" s="30" t="s">
-        <v>753</v>
+        <v>740</v>
       </c>
       <c r="C381" s="30" t="s">
-        <v>754</v>
+        <v>741</v>
       </c>
       <c r="D381" s="15" t="s">
         <v>17</v>
@@ -9990,7 +9919,7 @@
         <v>225</v>
       </c>
       <c r="C382" s="30" t="s">
-        <v>755</v>
+        <v>742</v>
       </c>
       <c r="D382" s="15" t="s">
         <v>1</v>
@@ -10004,7 +9933,7 @@
         <v>226</v>
       </c>
       <c r="C383" s="30" t="s">
-        <v>756</v>
+        <v>743</v>
       </c>
       <c r="D383" s="15" t="s">
         <v>0</v>
@@ -10018,13 +9947,13 @@
         <v>227</v>
       </c>
       <c r="C384" s="30" t="s">
-        <v>757</v>
+        <v>744</v>
       </c>
       <c r="D384" s="15" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="385" spans="1:4" ht="77.5" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:4" ht="62" x14ac:dyDescent="0.35">
       <c r="A385" s="10">
         <v>384</v>
       </c>
@@ -10032,7 +9961,7 @@
         <v>228</v>
       </c>
       <c r="C385" s="30" t="s">
-        <v>758</v>
+        <v>783</v>
       </c>
       <c r="D385" s="15" t="s">
         <v>1</v>
@@ -10046,7 +9975,7 @@
         <v>229</v>
       </c>
       <c r="C386" s="11" t="s">
-        <v>759</v>
+        <v>745</v>
       </c>
       <c r="D386" s="15" t="s">
         <v>17</v>
@@ -10060,7 +9989,7 @@
         <v>230</v>
       </c>
       <c r="C387" s="11" t="s">
-        <v>760</v>
+        <v>746</v>
       </c>
       <c r="D387" s="15" t="s">
         <v>20</v>
@@ -10074,7 +10003,7 @@
         <v>231</v>
       </c>
       <c r="C388" s="11" t="s">
-        <v>761</v>
+        <v>747</v>
       </c>
       <c r="D388" s="15" t="s">
         <v>17</v>
@@ -10085,10 +10014,10 @@
         <v>388</v>
       </c>
       <c r="B389" s="11" t="s">
-        <v>762</v>
+        <v>748</v>
       </c>
       <c r="C389" s="11" t="s">
-        <v>763</v>
+        <v>749</v>
       </c>
       <c r="D389" s="19" t="s">
         <v>1</v>
@@ -10099,10 +10028,10 @@
         <v>389</v>
       </c>
       <c r="B390" s="11" t="s">
-        <v>764</v>
+        <v>750</v>
       </c>
       <c r="C390" s="11" t="s">
-        <v>765</v>
+        <v>751</v>
       </c>
       <c r="D390" s="19" t="s">
         <v>1</v>
@@ -10116,7 +10045,7 @@
         <v>232</v>
       </c>
       <c r="C391" s="11" t="s">
-        <v>766</v>
+        <v>752</v>
       </c>
       <c r="D391" s="19" t="s">
         <v>1</v>

</xml_diff>